<commit_message>
data: migrar 22 lancamentos e 24 categorias do arquivo antigo para nova planilha
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -189,8 +188,12 @@
       <color rgb="006A1B9A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -262,6 +265,18 @@
         <fgColor rgb="00607D8B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+        <bgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -275,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -419,7 +434,7 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -437,6 +452,27 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="28" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -920,7 +956,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" customHeight="1">
+    <row r="3">
       <c r="A3" s="8" t="n"/>
       <c r="B3" s="8">
         <f>B2</f>
@@ -2229,380 +2265,796 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="52" t="inlineStr">
+      <c r="A2" s="63" t="inlineStr">
         <is>
           <t>Receita</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n">
-        <v>46208</v>
-      </c>
-      <c r="C2" s="52" t="inlineStr">
-        <is>
-          <t>Salário Will</t>
-        </is>
-      </c>
-      <c r="D2" s="52" t="inlineStr">
+      <c r="B2" s="64" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C2" s="65" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="E2" s="52" t="inlineStr">
+      <c r="D2" s="65" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="E2" s="63" t="inlineStr">
+        <is>
+          <t>Sá</t>
+        </is>
+      </c>
+      <c r="F2" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="66" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H2" s="63" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="63" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="B3" s="64" t="n">
+        <v>46206.625</v>
+      </c>
+      <c r="C3" s="65" t="inlineStr">
+        <is>
+          <t>13° Salário - Jun</t>
+        </is>
+      </c>
+      <c r="D3" s="65" t="inlineStr">
+        <is>
+          <t>13° Salário - Jun</t>
+        </is>
+      </c>
+      <c r="E3" s="63" t="inlineStr">
         <is>
           <t>Will</t>
         </is>
       </c>
-      <c r="F2" s="52" t="n">
+      <c r="F3" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="54" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H2" s="52" t="inlineStr">
+      <c r="G3" s="66" t="n">
+        <v>1687.8</v>
+      </c>
+      <c r="H3" s="63" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="52" t="inlineStr">
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="63" t="inlineStr">
         <is>
           <t>Receita</t>
         </is>
       </c>
-      <c r="B3" s="53" t="n">
-        <v>46208</v>
-      </c>
-      <c r="C3" s="52" t="inlineStr">
-        <is>
-          <t>Salário Sá</t>
-        </is>
-      </c>
-      <c r="D3" s="52" t="inlineStr">
+      <c r="B4" s="64" t="n">
+        <v>46206.625</v>
+      </c>
+      <c r="C4" s="65" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="E3" s="52" t="inlineStr">
+      <c r="D4" s="65" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="E4" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F4" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="66" t="n">
+        <v>966.37</v>
+      </c>
+      <c r="H4" s="63" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B5" s="64" t="n">
+        <v>46205.625</v>
+      </c>
+      <c r="C5" s="65" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="D5" s="65" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F5" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="66" t="n">
+        <v>164.62</v>
+      </c>
+      <c r="H5" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="n">
+        <v>46205.625</v>
+      </c>
+      <c r="C6" s="65" t="inlineStr">
+        <is>
+          <t>Cartão Will</t>
+        </is>
+      </c>
+      <c r="D6" s="65" t="inlineStr">
+        <is>
+          <t>Cartão Will</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="66" t="n">
+        <v>250</v>
+      </c>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="n">
+        <v>46206.625</v>
+      </c>
+      <c r="C7" s="65" t="inlineStr">
+        <is>
+          <t>Ração</t>
+        </is>
+      </c>
+      <c r="D7" s="65" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E7" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F7" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="66" t="n">
+        <v>189.9</v>
+      </c>
+      <c r="H7" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B8" s="64" t="n">
+        <v>46206.625</v>
+      </c>
+      <c r="C8" s="65" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D8" s="65" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="E8" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F8" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="66" t="n">
+        <v>24</v>
+      </c>
+      <c r="H8" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="n">
+        <v>46206.625</v>
+      </c>
+      <c r="C9" s="65" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="D9" s="65" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="E9" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F9" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="66" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="63" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="B10" s="64" t="n">
+        <v>46207.625</v>
+      </c>
+      <c r="C10" s="65" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D10" s="65" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="E10" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F10" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="66" t="n">
+        <v>190</v>
+      </c>
+      <c r="H10" s="63" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B11" s="64" t="n">
+        <v>46207.625</v>
+      </c>
+      <c r="C11" s="65" t="inlineStr">
+        <is>
+          <t>Ração</t>
+        </is>
+      </c>
+      <c r="D11" s="65" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E11" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F11" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="66" t="n">
+        <v>49.17</v>
+      </c>
+      <c r="H11" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B12" s="64" t="n">
+        <v>46207.625</v>
+      </c>
+      <c r="C12" s="65" t="inlineStr">
+        <is>
+          <t>Sem Parar - TAG</t>
+        </is>
+      </c>
+      <c r="D12" s="65" t="inlineStr">
+        <is>
+          <t>Sem Parar - TAG</t>
+        </is>
+      </c>
+      <c r="E12" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F12" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="66" t="n">
+        <v>129.7</v>
+      </c>
+      <c r="H12" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="63" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="B13" s="64" t="n">
+        <v>46207.625</v>
+      </c>
+      <c r="C13" s="65" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D13" s="65" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="E13" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F13" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="66" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="H13" s="63" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B14" s="64" t="n">
+        <v>46209.625</v>
+      </c>
+      <c r="C14" s="65" t="inlineStr">
+        <is>
+          <t>Condominio</t>
+        </is>
+      </c>
+      <c r="D14" s="65" t="inlineStr">
+        <is>
+          <t>Condominio</t>
+        </is>
+      </c>
+      <c r="E14" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F14" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="66" t="n">
+        <v>353.85</v>
+      </c>
+      <c r="H14" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B15" s="64" t="n">
+        <v>46209.625</v>
+      </c>
+      <c r="C15" s="65" t="inlineStr">
+        <is>
+          <t>Aluguel</t>
+        </is>
+      </c>
+      <c r="D15" s="65" t="inlineStr">
+        <is>
+          <t>Aluguel</t>
+        </is>
+      </c>
+      <c r="E15" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F15" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="66" t="n">
+        <v>1713.65</v>
+      </c>
+      <c r="H15" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B16" s="64" t="n">
+        <v>46209.625</v>
+      </c>
+      <c r="C16" s="65" t="inlineStr">
+        <is>
+          <t>Gás</t>
+        </is>
+      </c>
+      <c r="D16" s="65" t="inlineStr">
+        <is>
+          <t>Gás</t>
+        </is>
+      </c>
+      <c r="E16" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F16" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="66" t="n">
+        <v>23.61</v>
+      </c>
+      <c r="H16" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B17" s="64" t="n">
+        <v>46209.625</v>
+      </c>
+      <c r="C17" s="65" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="D17" s="65" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="E17" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F17" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="66" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="H17" s="63" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="63" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="B18" s="64" t="n">
+        <v>46218.625</v>
+      </c>
+      <c r="C18" s="65" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="D18" s="65" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="E18" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F18" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="66" t="n">
+        <v>1350</v>
+      </c>
+      <c r="H18" s="63" t="inlineStr">
+        <is>
+          <t>A Receber</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="63" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="B19" s="64" t="n">
+        <v>46218.625</v>
+      </c>
+      <c r="C19" s="65" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="D19" s="65" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
+      <c r="E19" s="63" t="inlineStr">
         <is>
           <t>Sá</t>
         </is>
       </c>
-      <c r="F3" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="54" t="n">
-        <v>3800</v>
-      </c>
-      <c r="H3" s="52" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="F19" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="66" t="n">
+        <v>1190</v>
+      </c>
+      <c r="H19" s="63" t="inlineStr">
+        <is>
+          <t>A Receber</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="63" t="inlineStr">
         <is>
           <t>Despesa</t>
         </is>
       </c>
-      <c r="B4" s="53" t="n">
-        <v>46206</v>
-      </c>
-      <c r="C4" s="52" t="inlineStr">
-        <is>
-          <t>Aluguel</t>
-        </is>
-      </c>
-      <c r="D4" s="52" t="inlineStr">
-        <is>
-          <t>Aluguel</t>
-        </is>
-      </c>
-      <c r="E4" s="52" t="inlineStr">
+      <c r="B20" s="64" t="n">
+        <v>46218.625</v>
+      </c>
+      <c r="C20" s="65" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="D20" s="65" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="E20" s="63" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="F4" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="54" t="n">
-        <v>1800</v>
-      </c>
-      <c r="H4" s="52" t="inlineStr">
-        <is>
-          <t>Pago</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="52" t="inlineStr">
+      <c r="F20" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="66" t="n">
+        <v>145</v>
+      </c>
+      <c r="H20" s="63" t="inlineStr">
+        <is>
+          <t>A Pagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="63" t="inlineStr">
         <is>
           <t>Despesa</t>
         </is>
       </c>
-      <c r="B5" s="53" t="n">
-        <v>46213</v>
-      </c>
-      <c r="C5" s="52" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="D5" s="52" t="inlineStr">
-        <is>
-          <t>Celular</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="B21" s="64" t="n">
+        <v>46218.625</v>
+      </c>
+      <c r="C21" s="65" t="inlineStr">
+        <is>
+          <t>Cartão Will</t>
+        </is>
+      </c>
+      <c r="D21" s="65" t="inlineStr">
+        <is>
+          <t>Cartão Will</t>
+        </is>
+      </c>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>Will</t>
+        </is>
+      </c>
+      <c r="F21" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="66" t="n">
+        <v>484.47</v>
+      </c>
+      <c r="H21" s="63" t="inlineStr">
+        <is>
+          <t>A Pagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="63" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="B22" s="64" t="n">
+        <v>46209.625</v>
+      </c>
+      <c r="C22" s="65" t="inlineStr">
+        <is>
+          <t>Gás</t>
+        </is>
+      </c>
+      <c r="D22" s="65" t="inlineStr">
+        <is>
+          <t>Gás</t>
+        </is>
+      </c>
+      <c r="E22" s="63" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="F5" s="52" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="54" t="n">
-        <v>150</v>
-      </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="F22" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="66" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="H22" s="63" t="inlineStr">
         <is>
           <t>A Pagar</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="52" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="63" t="inlineStr">
         <is>
           <t>Despesa</t>
         </is>
       </c>
-      <c r="B6" s="53" t="n">
-        <v>46218</v>
-      </c>
-      <c r="C6" s="52" t="inlineStr">
-        <is>
-          <t>Fatura Will</t>
-        </is>
-      </c>
-      <c r="D6" s="52" t="inlineStr">
-        <is>
-          <t>Cartões</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="inlineStr">
-        <is>
-          <t>Will</t>
-        </is>
-      </c>
-      <c r="F6" s="52" t="n">
+      <c r="B23" s="64" t="n">
+        <v>46218.625</v>
+      </c>
+      <c r="C23" s="65" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="D23" s="65" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="54" t="n">
-        <v>900</v>
-      </c>
-      <c r="H6" s="52" t="inlineStr">
+      <c r="G23" s="66" t="n">
+        <v>130</v>
+      </c>
+      <c r="H23" s="63" t="inlineStr">
         <is>
           <t>A Pagar</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t>Receita</t>
-        </is>
-      </c>
-      <c r="B7" s="53" t="n">
-        <v>46223</v>
-      </c>
-      <c r="C7" s="52" t="inlineStr">
-        <is>
-          <t>Renda Extra</t>
-        </is>
-      </c>
-      <c r="D7" s="52" t="inlineStr">
-        <is>
-          <t>Renda Extra</t>
-        </is>
-      </c>
-      <c r="E7" s="52" t="inlineStr">
-        <is>
-          <t>Will</t>
-        </is>
-      </c>
-      <c r="F7" s="52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="54" t="n">
-        <v>500</v>
-      </c>
-      <c r="H7" s="52" t="inlineStr">
-        <is>
-          <t>A Receber</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="55" t="n"/>
-      <c r="B8" s="55" t="n"/>
-      <c r="C8" s="55" t="n"/>
-      <c r="D8" s="55" t="n"/>
-      <c r="E8" s="55" t="n"/>
-      <c r="F8" s="55" t="n"/>
-      <c r="G8" s="55" t="n"/>
-      <c r="H8" s="55" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="55" t="n"/>
-      <c r="B9" s="55" t="n"/>
-      <c r="C9" s="55" t="n"/>
-      <c r="D9" s="55" t="n"/>
-      <c r="E9" s="55" t="n"/>
-      <c r="F9" s="55" t="n"/>
-      <c r="G9" s="55" t="n"/>
-      <c r="H9" s="55" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="55" t="n"/>
-      <c r="B10" s="55" t="n"/>
-      <c r="C10" s="55" t="n"/>
-      <c r="D10" s="55" t="n"/>
-      <c r="E10" s="55" t="n"/>
-      <c r="F10" s="55" t="n"/>
-      <c r="G10" s="55" t="n"/>
-      <c r="H10" s="55" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="55" t="n"/>
-      <c r="B11" s="55" t="n"/>
-      <c r="C11" s="55" t="n"/>
-      <c r="D11" s="55" t="n"/>
-      <c r="E11" s="55" t="n"/>
-      <c r="F11" s="55" t="n"/>
-      <c r="G11" s="55" t="n"/>
-      <c r="H11" s="55" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="55" t="n"/>
-      <c r="B12" s="55" t="n"/>
-      <c r="C12" s="55" t="n"/>
-      <c r="D12" s="55" t="n"/>
-      <c r="E12" s="55" t="n"/>
-      <c r="F12" s="55" t="n"/>
-      <c r="G12" s="55" t="n"/>
-      <c r="H12" s="55" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="55" t="n"/>
-      <c r="B13" s="55" t="n"/>
-      <c r="C13" s="55" t="n"/>
-      <c r="D13" s="55" t="n"/>
-      <c r="E13" s="55" t="n"/>
-      <c r="F13" s="55" t="n"/>
-      <c r="G13" s="55" t="n"/>
-      <c r="H13" s="55" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="55" t="n"/>
-      <c r="B14" s="55" t="n"/>
-      <c r="C14" s="55" t="n"/>
-      <c r="D14" s="55" t="n"/>
-      <c r="E14" s="55" t="n"/>
-      <c r="F14" s="55" t="n"/>
-      <c r="G14" s="55" t="n"/>
-      <c r="H14" s="55" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="55" t="n"/>
-      <c r="B15" s="55" t="n"/>
-      <c r="C15" s="55" t="n"/>
-      <c r="D15" s="55" t="n"/>
-      <c r="E15" s="55" t="n"/>
-      <c r="F15" s="55" t="n"/>
-      <c r="G15" s="55" t="n"/>
-      <c r="H15" s="55" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="55" t="n"/>
-      <c r="B16" s="55" t="n"/>
-      <c r="C16" s="55" t="n"/>
-      <c r="D16" s="55" t="n"/>
-      <c r="E16" s="55" t="n"/>
-      <c r="F16" s="55" t="n"/>
-      <c r="G16" s="55" t="n"/>
-      <c r="H16" s="55" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="55" t="n"/>
-      <c r="B17" s="55" t="n"/>
-      <c r="C17" s="55" t="n"/>
-      <c r="D17" s="55" t="n"/>
-      <c r="E17" s="55" t="n"/>
-      <c r="F17" s="55" t="n"/>
-      <c r="G17" s="55" t="n"/>
-      <c r="H17" s="55" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="55" t="n"/>
-      <c r="B18" s="55" t="n"/>
-      <c r="C18" s="55" t="n"/>
-      <c r="D18" s="55" t="n"/>
-      <c r="E18" s="55" t="n"/>
-      <c r="F18" s="55" t="n"/>
-      <c r="G18" s="55" t="n"/>
-      <c r="H18" s="55" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="55" t="n"/>
-      <c r="B19" s="55" t="n"/>
-      <c r="C19" s="55" t="n"/>
-      <c r="D19" s="55" t="n"/>
-      <c r="E19" s="55" t="n"/>
-      <c r="F19" s="55" t="n"/>
-      <c r="G19" s="55" t="n"/>
-      <c r="H19" s="55" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="55" t="n"/>
-      <c r="B20" s="55" t="n"/>
-      <c r="C20" s="55" t="n"/>
-      <c r="D20" s="55" t="n"/>
-      <c r="E20" s="55" t="n"/>
-      <c r="F20" s="55" t="n"/>
-      <c r="G20" s="55" t="n"/>
-      <c r="H20" s="55" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="55" t="n"/>
-      <c r="B21" s="55" t="n"/>
-      <c r="C21" s="55" t="n"/>
-      <c r="D21" s="55" t="n"/>
-      <c r="E21" s="55" t="n"/>
-      <c r="F21" s="55" t="n"/>
-      <c r="G21" s="55" t="n"/>
-      <c r="H21" s="55" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="55" t="n"/>
-      <c r="B22" s="55" t="n"/>
-      <c r="C22" s="55" t="n"/>
-      <c r="D22" s="55" t="n"/>
-      <c r="E22" s="55" t="n"/>
-      <c r="F22" s="55" t="n"/>
-      <c r="G22" s="55" t="n"/>
-      <c r="H22" s="55" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="55" t="n"/>
-      <c r="B23" s="55" t="n"/>
-      <c r="C23" s="55" t="n"/>
-      <c r="D23" s="55" t="n"/>
-      <c r="E23" s="55" t="n"/>
-      <c r="F23" s="55" t="n"/>
-      <c r="G23" s="55" t="n"/>
-      <c r="H23" s="55" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="55" t="n"/>
@@ -7696,7 +8148,7 @@
       <c r="B2" s="8" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="61" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
@@ -7704,155 +8156,187 @@
       <c r="B3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>13° Salário - Dez</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>PLR</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t>Férias</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>Renda Extra</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="59" t="inlineStr">
-        <is>
-          <t>13° Salário</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="52" t="inlineStr">
-        <is>
-          <t>PLR</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="59" t="inlineStr">
-        <is>
-          <t>Férias</t>
-        </is>
-      </c>
       <c r="B7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="52" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="62" t="inlineStr">
+        <is>
+          <t>Condominio</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>Cartão Will</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="62" t="inlineStr">
+        <is>
+          <t>Cartão Sá</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>Gás</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>Unha mão</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="62" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>Aluguel</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="59" t="inlineStr">
+      <c r="B17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="62" t="inlineStr">
+        <is>
+          <t>Farmácia</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="62" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="52" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="59" t="inlineStr">
-        <is>
-          <t>Saúde</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="52" t="inlineStr">
-        <is>
-          <t>Lazer</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="59" t="inlineStr">
-        <is>
-          <t>Cartões</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="52" t="inlineStr">
-        <is>
-          <t>Celular</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="59" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="52" t="inlineStr">
-        <is>
-          <t>Luz</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="59" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="52" t="inlineStr">
+      <c r="B21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
         <is>
           <t>Outros</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n"/>
-      <c r="B20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n"/>
       <c r="B22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n"/>
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>13° Salário - Jun</t>
+        </is>
+      </c>
       <c r="B23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="n"/>
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>Adiantamento</t>
+        </is>
+      </c>
       <c r="B24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n"/>
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>Sem Parar - TAG</t>
+        </is>
+      </c>
       <c r="B25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n"/>
+      <c r="A26" s="62" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
       <c r="B26" s="8" t="n"/>
     </row>
     <row r="27">

</xml_diff>

<commit_message>
fix: corrigir ranges das formulas SUMPRODUCT no dropdown de visualizacao
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="B5" s="111">
-        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*(Lancamentos!$F$2:$A$487=1)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*(Lancamentos!$F$2:$A$487=2)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*Lancamentos!$G$2:$A$487)),0)</f>
+        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=1)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=2)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487)),0)</f>
         <v/>
       </c>
       <c r="C5" s="112" t="n"/>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="G5" s="114">
-        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*(Lancamentos!$F$2:$A$487=1)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*(Lancamentos!$F$2:$A$487=2)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$A$487)=$B$2)*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*Lancamentos!$G$2:$A$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$A$487)=$B$3)*Lancamentos!$G$2:$A$487)),0)</f>
+        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=1)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=2)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487)),0)</f>
         <v/>
       </c>
       <c r="H5" s="113" t="n"/>

</xml_diff>

<commit_message>
fix: usar IF simples no dropdown apontando para celulas RESUMO (B11/C11/D11)
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="B5" s="111">
-        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=1)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=2)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487)),0)</f>
+        <f>IFERROR(IF($I$3="C1",B11,IF($I$3="C2",C11,IF($I$3="Anual",SUMPRODUCT((Lancamentos!$A$2:$A$487="Receita")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),D11))),0)</f>
         <v/>
       </c>
       <c r="C5" s="112" t="n"/>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="G5" s="114">
-        <f>IFERROR(CHOOSE(MATCH($I$3,{"C1","C2","C1+C2","Anual"},0),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=1)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*(Lancamentos!$F$2:$F$487=2)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(MONTH(Lancamentos!$B$2:$B$487)=$B$2)*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487)),0)</f>
+        <f>IFERROR(IF($I$3="C1",B12,IF($I$3="C2",C12,IF($I$3="Anual",SUMPRODUCT((Lancamentos!$A$2:$A$487="Despesa")*(Lancamentos!$B$2:$B$487&lt;&gt;"")*(YEAR(Lancamentos!$B$2:$B$487)=$B$3)*Lancamentos!$G$2:$G$487),D12))),0)</f>
         <v/>
       </c>
       <c r="H5" s="113" t="n"/>

</xml_diff>

<commit_message>
feat: adicionar aba Planejamento de Viagem com calculadora de combustivel, hospedagem, alimentacao e resumo total
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Investimentos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cartoes" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="Config" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Planejamento Viagem" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lancamentos'!$A$1:$H$23</definedName>
@@ -19,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
@@ -27,8 +28,9 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="dd/MM/yyyy HH:mm"/>
     <numFmt numFmtId="170" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="65">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -272,8 +274,166 @@
       <color rgb="00F39C12"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002980B9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0016A085"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002980B9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00CC6600"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002980B9"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002980B9"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0027AE60"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E8449"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0027AE60"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="008E44AD"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="008E44AD"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0027AE60"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="008E44AD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00F1C40F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0027AE60"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -355,6 +515,76 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016A085"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E67E22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002980B9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0027AE60"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008E44AD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9F0FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8DAEF"/>
       </patternFill>
     </fill>
   </fills>
@@ -709,7 +939,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="192">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -947,6 +1177,183 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="48" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="48" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="45" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="51" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="52" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="53" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="53" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="53" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="55" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="45" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="57" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="48" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="41" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="61" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="62" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="37" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="64" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2886,11 +3293,11 @@
     <row r="1000" ht="15.75" customHeight="1" s="101"/>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A20:B20"/>
+    <mergeCell ref="J3:K3"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="D3:G3"/>
-    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="A19:K19"/>
@@ -19174,4 +19581,635 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0016A085"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="101" min="1" max="1"/>
+    <col width="22" customWidth="1" style="101" min="2" max="2"/>
+    <col width="16" customWidth="1" style="101" min="3" max="3"/>
+    <col width="16" customWidth="1" style="101" min="4" max="4"/>
+    <col width="16" customWidth="1" style="101" min="5" max="5"/>
+    <col width="16" customWidth="1" style="101" min="6" max="6"/>
+    <col width="16" customWidth="1" style="101" min="7" max="7"/>
+    <col width="3" customWidth="1" style="101" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1" s="101">
+      <c r="B1" s="125" t="inlineStr">
+        <is>
+          <t>✈️  PLANEJAMENTO DE VIAGEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1" s="101"/>
+    <row r="3" ht="26" customHeight="1" s="101">
+      <c r="B3" s="126" t="inlineStr">
+        <is>
+          <t>📋  DADOS DA VIAGEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" s="101">
+      <c r="B4" s="127" t="inlineStr">
+        <is>
+          <t>Nome da Viagem</t>
+        </is>
+      </c>
+      <c r="C4" s="128" t="inlineStr"/>
+      <c r="D4" s="129" t="inlineStr">
+        <is>
+          <t>Ex: Viagem a Floripa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="101">
+      <c r="B5" s="130" t="inlineStr">
+        <is>
+          <t>Data de Saída</t>
+        </is>
+      </c>
+      <c r="C5" s="128" t="n"/>
+      <c r="D5" s="131" t="inlineStr">
+        <is>
+          <t>← preencha a data de saída</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="101">
+      <c r="B6" s="127" t="inlineStr">
+        <is>
+          <t>Data de Retorno</t>
+        </is>
+      </c>
+      <c r="C6" s="128" t="n"/>
+      <c r="D6" s="132">
+        <f>IF(AND(C5&lt;&gt;"",C6&lt;&gt;""),TEXT(C6-C5,"0")&amp;" dias","— informe as datas")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="101">
+      <c r="B7" s="130" t="inlineStr">
+        <is>
+          <t>Nº de Pessoas</t>
+        </is>
+      </c>
+      <c r="C7" s="128" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="133" t="n"/>
+      <c r="E7" s="133" t="n"/>
+      <c r="F7" s="133" t="n"/>
+      <c r="G7" s="133" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" s="101">
+      <c r="B8" s="127" t="inlineStr">
+        <is>
+          <t>Orçamento Total (R$)</t>
+        </is>
+      </c>
+      <c r="C8" s="134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="135" t="n"/>
+      <c r="E8" s="135" t="n"/>
+      <c r="F8" s="135" t="n"/>
+      <c r="G8" s="135" t="n"/>
+    </row>
+    <row r="9" ht="10" customHeight="1" s="101"/>
+    <row r="10" ht="26" customHeight="1" s="101">
+      <c r="B10" s="136" t="inlineStr">
+        <is>
+          <t>⛽  CALCULADORA DE COMBUSTÍVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" s="101">
+      <c r="B11" s="137" t="inlineStr">
+        <is>
+          <t>Distância total (km)</t>
+        </is>
+      </c>
+      <c r="C11" s="138" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="133" t="n"/>
+      <c r="E11" s="131" t="inlineStr">
+        <is>
+          <t>Ida + volta. Ex: SP→Floripa = 600km × 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" s="101">
+      <c r="B12" s="139" t="inlineStr">
+        <is>
+          <t>Consumo do carro (km/L)</t>
+        </is>
+      </c>
+      <c r="C12" s="140" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="141" t="n"/>
+      <c r="E12" s="142" t="inlineStr">
+        <is>
+          <t>Consulte o manual do veículo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="101">
+      <c r="B13" s="137" t="inlineStr">
+        <is>
+          <t>Tipo de combustível</t>
+        </is>
+      </c>
+      <c r="C13" s="143" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+      <c r="D13" s="133" t="n"/>
+      <c r="E13" s="131" t="inlineStr">
+        <is>
+          <t>Gasolina / Etanol / Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="101">
+      <c r="B14" s="139" t="inlineStr">
+        <is>
+          <t>Preço do combustível (R$/L)</t>
+        </is>
+      </c>
+      <c r="C14" s="144" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D14" s="141" t="n"/>
+      <c r="E14" s="142" t="inlineStr">
+        <is>
+          <t>← insira o preço atual (veja nota abaixo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" s="101">
+      <c r="B15" s="145" t="inlineStr">
+        <is>
+          <t>— Litros necessários</t>
+        </is>
+      </c>
+      <c r="C15" s="146">
+        <f>IFERROR(C11/C12,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="133" t="n"/>
+      <c r="E15" s="131">
+        <f> distância ÷ consumo</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="101">
+      <c r="B16" s="147" t="inlineStr">
+        <is>
+          <t>— Custo total combustível</t>
+        </is>
+      </c>
+      <c r="C16" s="148">
+        <f>IFERROR(C15*C14,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="141" t="n"/>
+      <c r="E16" s="142">
+        <f> litros × preço</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="101">
+      <c r="B17" s="145" t="inlineStr">
+        <is>
+          <t>— Custo por pessoa</t>
+        </is>
+      </c>
+      <c r="C17" s="148">
+        <f>IFERROR(C16/C7,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="133" t="n"/>
+      <c r="E17" s="131">
+        <f> custo total ÷ nº pessoas (C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1" s="101">
+      <c r="B18" s="149" t="inlineStr">
+        <is>
+          <t>💡 Preço do combustível: consulte https://www.gov.br/anp (média semanal por estado) ou apps como Waze / Meu Combustível / Postos da Cidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="10" customHeight="1" s="101"/>
+    <row r="20" ht="26" customHeight="1" s="101">
+      <c r="B20" s="150" t="inlineStr">
+        <is>
+          <t>🏨  HOSPEDAGEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="101">
+      <c r="B21" s="151" t="inlineStr">
+        <is>
+          <t>Local / Acomodação</t>
+        </is>
+      </c>
+      <c r="C21" s="151" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="D21" s="151" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E21" s="151" t="inlineStr">
+        <is>
+          <t>Noites</t>
+        </is>
+      </c>
+      <c r="F21" s="151" t="inlineStr">
+        <is>
+          <t>R$/Noite</t>
+        </is>
+      </c>
+      <c r="G21" s="151" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="101">
+      <c r="B22" s="152" t="n"/>
+      <c r="C22" s="152" t="n"/>
+      <c r="D22" s="152" t="n"/>
+      <c r="E22" s="153">
+        <f>IFERROR(D22-C22,0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="154" t="n"/>
+      <c r="G22" s="155">
+        <f>IFERROR(E22*F22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" s="101">
+      <c r="B23" s="156" t="n"/>
+      <c r="C23" s="156" t="n"/>
+      <c r="D23" s="156" t="n"/>
+      <c r="E23" s="157">
+        <f>IFERROR(D23-C23,0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="158" t="n"/>
+      <c r="G23" s="159">
+        <f>IFERROR(E23*F23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" s="101">
+      <c r="B24" s="152" t="n"/>
+      <c r="C24" s="152" t="n"/>
+      <c r="D24" s="152" t="n"/>
+      <c r="E24" s="153">
+        <f>IFERROR(D24-C24,0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="154" t="n"/>
+      <c r="G24" s="155">
+        <f>IFERROR(E24*F24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" s="101">
+      <c r="B25" s="156" t="n"/>
+      <c r="C25" s="156" t="n"/>
+      <c r="D25" s="156" t="n"/>
+      <c r="E25" s="157">
+        <f>IFERROR(D25-C25,0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="158" t="n"/>
+      <c r="G25" s="159">
+        <f>IFERROR(E25*F25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" s="101">
+      <c r="B26" s="152" t="n"/>
+      <c r="C26" s="152" t="n"/>
+      <c r="D26" s="152" t="n"/>
+      <c r="E26" s="153">
+        <f>IFERROR(D26-C26,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="154" t="n"/>
+      <c r="G26" s="155">
+        <f>IFERROR(E26*F26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="101">
+      <c r="B27" s="160" t="inlineStr">
+        <is>
+          <t>TOTAL HOSPEDAGEM</t>
+        </is>
+      </c>
+      <c r="G27" s="161">
+        <f>SUM(G22:G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="10" customHeight="1" s="101"/>
+    <row r="29" ht="26" customHeight="1" s="101">
+      <c r="B29" s="162" t="inlineStr">
+        <is>
+          <t>🍽️  ALIMENTAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="101">
+      <c r="B30" s="163" t="inlineStr">
+        <is>
+          <t>Custo estimado por pessoa/dia (R$)</t>
+        </is>
+      </c>
+      <c r="C30" s="164" t="n">
+        <v>80</v>
+      </c>
+      <c r="D30" s="135" t="n"/>
+      <c r="E30" s="135" t="n"/>
+      <c r="F30" s="135" t="n"/>
+      <c r="G30" s="135" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1" s="101">
+      <c r="B31" s="137" t="inlineStr">
+        <is>
+          <t>Número de dias</t>
+        </is>
+      </c>
+      <c r="C31" s="165">
+        <f>IFERROR(C6-C5,0)</f>
+        <v/>
+      </c>
+      <c r="D31" s="133" t="n"/>
+      <c r="E31" s="133" t="n"/>
+      <c r="F31" s="133" t="n"/>
+      <c r="G31" s="133" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="101">
+      <c r="B32" s="163" t="inlineStr">
+        <is>
+          <t>Número de pessoas</t>
+        </is>
+      </c>
+      <c r="C32" s="166">
+        <f>C7</f>
+        <v/>
+      </c>
+      <c r="D32" s="135" t="n"/>
+      <c r="E32" s="135" t="n"/>
+      <c r="F32" s="135" t="n"/>
+      <c r="G32" s="135" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="101">
+      <c r="B33" s="167" t="inlineStr">
+        <is>
+          <t>— TOTAL ALIMENTAÇÃO</t>
+        </is>
+      </c>
+      <c r="C33" s="168">
+        <f>IFERROR(C30*C31*C32,0)</f>
+        <v/>
+      </c>
+      <c r="D33" s="169" t="n"/>
+      <c r="E33" s="169" t="n"/>
+      <c r="F33" s="169" t="n"/>
+      <c r="G33" s="169" t="n"/>
+    </row>
+    <row r="34" ht="10" customHeight="1" s="101"/>
+    <row r="35" ht="26" customHeight="1" s="101">
+      <c r="B35" s="170" t="inlineStr">
+        <is>
+          <t>🎡  PASSEIOS E OUTROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" s="101">
+      <c r="B36" s="151" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="C36" s="151" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D36" s="171" t="n"/>
+      <c r="E36" s="171" t="n"/>
+      <c r="F36" s="171" t="n"/>
+      <c r="G36" s="151" t="inlineStr">
+        <is>
+          <t>Valor (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" s="101">
+      <c r="B37" s="172" t="n"/>
+      <c r="C37" s="172" t="n"/>
+      <c r="D37" s="172" t="n"/>
+      <c r="E37" s="172" t="n"/>
+      <c r="F37" s="172" t="n"/>
+      <c r="G37" s="173" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1" s="101">
+      <c r="B38" s="133" t="n"/>
+      <c r="C38" s="133" t="n"/>
+      <c r="D38" s="133" t="n"/>
+      <c r="E38" s="133" t="n"/>
+      <c r="F38" s="133" t="n"/>
+      <c r="G38" s="174" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1" s="101">
+      <c r="B39" s="172" t="n"/>
+      <c r="C39" s="172" t="n"/>
+      <c r="D39" s="172" t="n"/>
+      <c r="E39" s="172" t="n"/>
+      <c r="F39" s="172" t="n"/>
+      <c r="G39" s="173" t="n"/>
+    </row>
+    <row r="40" ht="20" customHeight="1" s="101">
+      <c r="B40" s="133" t="n"/>
+      <c r="C40" s="133" t="n"/>
+      <c r="D40" s="133" t="n"/>
+      <c r="E40" s="133" t="n"/>
+      <c r="F40" s="133" t="n"/>
+      <c r="G40" s="174" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="101">
+      <c r="B41" s="172" t="n"/>
+      <c r="C41" s="172" t="n"/>
+      <c r="D41" s="172" t="n"/>
+      <c r="E41" s="172" t="n"/>
+      <c r="F41" s="172" t="n"/>
+      <c r="G41" s="173" t="n"/>
+    </row>
+    <row r="42" ht="20" customHeight="1" s="101">
+      <c r="B42" s="133" t="n"/>
+      <c r="C42" s="133" t="n"/>
+      <c r="D42" s="133" t="n"/>
+      <c r="E42" s="133" t="n"/>
+      <c r="F42" s="133" t="n"/>
+      <c r="G42" s="174" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1" s="101">
+      <c r="B43" s="175" t="inlineStr">
+        <is>
+          <t>TOTAL OUTROS</t>
+        </is>
+      </c>
+      <c r="G43" s="176">
+        <f>SUM(G37:G42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="10" customHeight="1" s="101"/>
+    <row r="45" ht="26" customHeight="1" s="101">
+      <c r="B45" s="177" t="inlineStr">
+        <is>
+          <t>💰  RESUMO TOTAL DA VIAGEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1" s="101">
+      <c r="B46" s="178" t="inlineStr">
+        <is>
+          <t>⛽ Combustível</t>
+        </is>
+      </c>
+      <c r="G46" s="179">
+        <f>C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1" s="101">
+      <c r="B47" s="180" t="inlineStr">
+        <is>
+          <t>🏨 Hospedagem</t>
+        </is>
+      </c>
+      <c r="G47" s="181">
+        <f>G27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1" s="101">
+      <c r="B48" s="182" t="inlineStr">
+        <is>
+          <t>🍽️ Alimentação</t>
+        </is>
+      </c>
+      <c r="G48" s="183">
+        <f>C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1" s="101">
+      <c r="B49" s="184" t="inlineStr">
+        <is>
+          <t>🎡 Outros</t>
+        </is>
+      </c>
+      <c r="G49" s="185">
+        <f>G43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="36" customHeight="1" s="101">
+      <c r="B50" s="186" t="inlineStr">
+        <is>
+          <t>🧳 TOTAL DA VIAGEM</t>
+        </is>
+      </c>
+      <c r="G50" s="187">
+        <f>SUM(G46:G49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" s="101">
+      <c r="B51" s="188" t="inlineStr">
+        <is>
+          <t>👤 Total por pessoa</t>
+        </is>
+      </c>
+      <c r="G51" s="189">
+        <f>IFERROR(G50/C7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1" s="101">
+      <c r="B52" s="190">
+        <f>IF(C8-G50&gt;=0,"✅ Sobra do orçamento","⚠️ Estouro do orçamento")</f>
+        <v/>
+      </c>
+      <c r="G52" s="191">
+        <f>C8-G50</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="D4:G4"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C37:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Ingresso,Passeio,Transporte,Compras,Emergência,Outro"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C37:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Ingresso,Passeio,Transporte,Compras,Emergência,Outro"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adicionar aba Compras e Metas com calculadora de poupanca e comparador a vista vs parcelado
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Cartoes" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="Config" sheetId="5" state="hidden" r:id="rId5"/>
     <sheet name="Planejamento Viagem" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Compras &amp; Metas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lancamentos'!$A$1:$H$23</definedName>
@@ -20,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
@@ -29,8 +30,12 @@
     <numFmt numFmtId="169" formatCode="dd/MM/yyyy HH:mm"/>
     <numFmt numFmtId="170" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="0 &quot;meses&quot;"/>
+    <numFmt numFmtId="173" formatCode="MMM/YYYY"/>
+    <numFmt numFmtId="174" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="65">
+  <fonts count="81">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -432,8 +437,100 @@
       <color rgb="0027AE60"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001A5276"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E74C3C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E86C1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0016A085"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002E86C1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00E74C3C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002980B9"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002980B9"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E74C3C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="007F8C8D"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="29">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -585,6 +682,51 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8DAEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E86C1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A5276"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -939,7 +1081,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="192">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1353,6 +1495,157 @@
     </xf>
     <xf numFmtId="4" fontId="64" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="66" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="63" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="67" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="68" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="70" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="70" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="72" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="69" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="74" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="44" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="75" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="76" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="74" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="44" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="75" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="76" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="78" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="78" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="66" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="66" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="79" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="80" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -20212,4 +20505,588 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E74C3C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="101" min="1" max="1"/>
+    <col width="20" customWidth="1" style="101" min="2" max="2"/>
+    <col width="8" customWidth="1" style="101" min="3" max="3"/>
+    <col width="8" customWidth="1" style="101" min="4" max="4"/>
+    <col width="3" customWidth="1" style="101" min="5" max="5"/>
+    <col width="16" customWidth="1" style="101" min="6" max="6"/>
+    <col width="8" customWidth="1" style="101" min="7" max="7"/>
+    <col width="8" customWidth="1" style="101" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1" s="101">
+      <c r="A1" s="192" t="inlineStr">
+        <is>
+          <t>🛒  COMPRAS &amp; METAS FINANCEIRAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="10" customHeight="1" s="101"/>
+    <row r="3" ht="28" customHeight="1" s="101">
+      <c r="A3" s="193" t="inlineStr">
+        <is>
+          <t>🎯  CALCULADORA DE META — Quanto guardar por mês</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" s="101">
+      <c r="A4" s="194" t="inlineStr">
+        <is>
+          <t>Produto / Objetivo</t>
+        </is>
+      </c>
+      <c r="E4" s="195" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="101">
+      <c r="A5" s="194" t="inlineStr">
+        <is>
+          <t>Valor total necessário (R$)</t>
+        </is>
+      </c>
+      <c r="E5" s="196" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="101">
+      <c r="A6" s="197" t="inlineStr">
+        <is>
+          <t>Já tenho guardado (R$)</t>
+        </is>
+      </c>
+      <c r="E6" s="196" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="101">
+      <c r="A7" s="198" t="inlineStr">
+        <is>
+          <t>→ Quanto ainda falta (R$)</t>
+        </is>
+      </c>
+      <c r="E7" s="199">
+        <f>IFERROR(E5-E6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="10" customHeight="1" s="101">
+      <c r="A8" s="200" t="n"/>
+      <c r="B8" s="200" t="n"/>
+      <c r="C8" s="200" t="n"/>
+      <c r="D8" s="200" t="n"/>
+      <c r="E8" s="200" t="n"/>
+      <c r="F8" s="200" t="n"/>
+      <c r="G8" s="200" t="n"/>
+      <c r="H8" s="200" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1" s="101">
+      <c r="A9" s="201" t="inlineStr">
+        <is>
+          <t>📌 OPÇÃO A — Quero comprar em X meses</t>
+        </is>
+      </c>
+      <c r="E9" s="202" t="inlineStr">
+        <is>
+          <t>📌 OPÇÃO B — Consigo guardar X por mês</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="101">
+      <c r="A10" s="203" t="inlineStr">
+        <is>
+          <t>Quero comprar em (meses):</t>
+        </is>
+      </c>
+      <c r="C10" s="204" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="203" t="inlineStr">
+        <is>
+          <t>Consigo guardar por mês (R$):</t>
+        </is>
+      </c>
+      <c r="G10" s="205" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1" s="101">
+      <c r="A11" s="206" t="inlineStr">
+        <is>
+          <t>→ Guardar por mês:</t>
+        </is>
+      </c>
+      <c r="C11" s="207">
+        <f>IFERROR(E7/C10,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="206" t="inlineStr">
+        <is>
+          <t>→ Meses até a compra:</t>
+        </is>
+      </c>
+      <c r="G11" s="208">
+        <f>IFERROR(CEILING(E7/G10,1),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" s="101">
+      <c r="A12" s="209" t="inlineStr">
+        <is>
+          <t>→ Data estimada (Opção A):</t>
+        </is>
+      </c>
+      <c r="C12" s="210">
+        <f>IFERROR(EDATE(TODAY(),C10),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="209" t="inlineStr">
+        <is>
+          <t>→ Data estimada (Opção B):</t>
+        </is>
+      </c>
+      <c r="G12" s="211">
+        <f>IFERROR(EDATE(TODAY(),G11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="10" customHeight="1" s="101"/>
+    <row r="14" ht="26" customHeight="1" s="101">
+      <c r="A14" s="212" t="inlineStr">
+        <is>
+          <t>📋  LISTA DE METAS DE COMPRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" s="101">
+      <c r="A15" s="213" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B15" s="213" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C15" s="213" t="inlineStr">
+        <is>
+          <t>Valor (R$)</t>
+        </is>
+      </c>
+      <c r="D15" s="213" t="inlineStr">
+        <is>
+          <t>Guardado (R$)</t>
+        </is>
+      </c>
+      <c r="E15" s="213" t="inlineStr">
+        <is>
+          <t>Falta (R$)</t>
+        </is>
+      </c>
+      <c r="F15" s="213" t="inlineStr">
+        <is>
+          <t>Poupar/mês</t>
+        </is>
+      </c>
+      <c r="G15" s="213" t="inlineStr">
+        <is>
+          <t>Meses</t>
+        </is>
+      </c>
+      <c r="H15" s="213" t="inlineStr">
+        <is>
+          <t>Previsão</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="101">
+      <c r="A16" s="214" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="135" t="n"/>
+      <c r="C16" s="215" t="n"/>
+      <c r="D16" s="215" t="n"/>
+      <c r="E16" s="216">
+        <f>IFERROR(C16-D16,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="217">
+        <f>IFERROR(E16/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="218">
+        <f>IFERROR(CEILING(E16/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H16" s="219">
+        <f>IFERROR(EDATE(TODAY(),G16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="101">
+      <c r="A17" s="220" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="133" t="n"/>
+      <c r="C17" s="221" t="n"/>
+      <c r="D17" s="221" t="n"/>
+      <c r="E17" s="222">
+        <f>IFERROR(C17-D17,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="223">
+        <f>IFERROR(E17/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="224">
+        <f>IFERROR(CEILING(E17/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H17" s="225">
+        <f>IFERROR(EDATE(TODAY(),G17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" s="101">
+      <c r="A18" s="214" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="135" t="n"/>
+      <c r="C18" s="215" t="n"/>
+      <c r="D18" s="215" t="n"/>
+      <c r="E18" s="216">
+        <f>IFERROR(C18-D18,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="217">
+        <f>IFERROR(E18/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="218">
+        <f>IFERROR(CEILING(E18/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H18" s="219">
+        <f>IFERROR(EDATE(TODAY(),G18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" s="101">
+      <c r="A19" s="220" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="133" t="n"/>
+      <c r="C19" s="221" t="n"/>
+      <c r="D19" s="221" t="n"/>
+      <c r="E19" s="222">
+        <f>IFERROR(C19-D19,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="223">
+        <f>IFERROR(E19/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="224">
+        <f>IFERROR(CEILING(E19/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H19" s="225">
+        <f>IFERROR(EDATE(TODAY(),G19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" s="101">
+      <c r="A20" s="214" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="135" t="n"/>
+      <c r="C20" s="215" t="n"/>
+      <c r="D20" s="215" t="n"/>
+      <c r="E20" s="216">
+        <f>IFERROR(C20-D20,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="217">
+        <f>IFERROR(E20/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G20" s="218">
+        <f>IFERROR(CEILING(E20/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H20" s="219">
+        <f>IFERROR(EDATE(TODAY(),G20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="101">
+      <c r="A21" s="220" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="133" t="n"/>
+      <c r="C21" s="221" t="n"/>
+      <c r="D21" s="221" t="n"/>
+      <c r="E21" s="222">
+        <f>IFERROR(C21-D21,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="223">
+        <f>IFERROR(E21/C10,0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="224">
+        <f>IFERROR(CEILING(E21/G10,1),0)</f>
+        <v/>
+      </c>
+      <c r="H21" s="225">
+        <f>IFERROR(EDATE(TODAY(),G21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1" s="101"/>
+    <row r="24" ht="28" customHeight="1" s="101">
+      <c r="A24" s="226" t="inlineStr">
+        <is>
+          <t>💳  CALCULADORA: À VISTA vs PARCELADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14" customHeight="1" s="101">
+      <c r="A25" s="227" t="inlineStr">
+        <is>
+          <t>Preencha os campos em AZUL — o restante é calculado automaticamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" s="101">
+      <c r="A26" s="197" t="inlineStr">
+        <is>
+          <t>Produto / Descrição</t>
+        </is>
+      </c>
+      <c r="E26" s="228" t="inlineStr"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="101">
+      <c r="A27" s="229" t="inlineStr">
+        <is>
+          <t>Preço à VISTA (R$)</t>
+        </is>
+      </c>
+      <c r="E27" s="230" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" s="101">
+      <c r="A28" s="197" t="inlineStr">
+        <is>
+          <t>Desconto à vista (%)</t>
+        </is>
+      </c>
+      <c r="E28" s="231" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="101">
+      <c r="A29" s="232" t="inlineStr">
+        <is>
+          <t>→ Preço à vista c/ desconto</t>
+        </is>
+      </c>
+      <c r="E29" s="233">
+        <f>IFERROR(E27*(1-E28/100),E27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="101">
+      <c r="A30" s="197" t="inlineStr">
+        <is>
+          <t>Número de parcelas</t>
+        </is>
+      </c>
+      <c r="E30" s="234" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" s="101">
+      <c r="A31" s="229" t="inlineStr">
+        <is>
+          <t>Valor de cada parcela (R$)</t>
+        </is>
+      </c>
+      <c r="E31" s="230" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1" s="101">
+      <c r="A32" s="200" t="n"/>
+      <c r="B32" s="200" t="n"/>
+      <c r="C32" s="200" t="n"/>
+      <c r="D32" s="200" t="n"/>
+      <c r="E32" s="200" t="n"/>
+      <c r="F32" s="200" t="n"/>
+      <c r="G32" s="200" t="n"/>
+      <c r="H32" s="200" t="n"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" s="101">
+      <c r="A33" s="212" t="inlineStr">
+        <is>
+          <t>📊  ANÁLISE COMPARATIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" s="101">
+      <c r="A34" s="197" t="inlineStr">
+        <is>
+          <t>💵 Total pago à vista</t>
+        </is>
+      </c>
+      <c r="E34" s="235">
+        <f>IFERROR(E29,E27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" s="101">
+      <c r="A35" s="229" t="inlineStr">
+        <is>
+          <t>💳 Total pago parcelado</t>
+        </is>
+      </c>
+      <c r="E35" s="236">
+        <f>IFERROR(E30*E31,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" s="101">
+      <c r="A36" s="237" t="inlineStr">
+        <is>
+          <t>📈 Quanto a mais no parcelado (R$)</t>
+        </is>
+      </c>
+      <c r="E36" s="238">
+        <f>IFERROR(E35-E34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="101">
+      <c r="A37" s="237" t="inlineStr">
+        <is>
+          <t>📈 Quanto a mais no parcelado (%)</t>
+        </is>
+      </c>
+      <c r="E37" s="239">
+        <f>IFERROR((E35/E34-1)*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1" s="101">
+      <c r="A38" s="237" t="inlineStr">
+        <is>
+          <t>🔢 Taxa de juros mensal (RATE)</t>
+        </is>
+      </c>
+      <c r="E38" s="240">
+        <f>IFERROR(RATE(E30,-E31,E29)*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1" s="101">
+      <c r="A39" s="237" t="inlineStr">
+        <is>
+          <t>🔢 Taxa de juros anual equivalente</t>
+        </is>
+      </c>
+      <c r="E39" s="240">
+        <f>IFERROR(((1+E38/100)^12-1)*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="10" customHeight="1" s="101"/>
+    <row r="41" ht="40" customHeight="1" s="101">
+      <c r="A41" s="241">
+        <f>IFERROR(IF(E38&lt;=0,"⚠️ Preencha preço à vista e valor da parcela",
+IF(E38&lt;0.8,"✅ JUROS BAIXOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Parcelar pode valer se você investir a diferença",
+IF(E38&lt;1.5,"⚡ JUROS MODERADOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Prefira à vista se possível",
+IF(E38&lt;3,"🔴 JUROS ALTOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Compre À VISTA. Parcelado custa "&amp;TEXT(E36,"R$ #,##0.00")&amp;" a mais",
+"🚨 JUROS ABUSIVOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — NUNCA parcele nessas condições!")))),"Preencha os dados")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1" s="101">
+      <c r="A42" s="242" t="inlineStr">
+        <is>
+          <t>💡 Dica: Se os juros forem menores que o rendimento da sua reserva (ex: CDB/Tesouro ~0,8%/mês), pode valer guardar o dinheiro e parcelar. Mas se não tiver disciplina, pague à vista.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="54">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="E39:H39"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E35:H35"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E38:H38"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="E29:H29"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="E34:H34"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E30:H30"/>
+    <mergeCell ref="E27:H27"/>
+    <mergeCell ref="E36:H36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adicionar dicas do destino com Nominatim + Overpass + Wikipedia + links Google Maps
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -1081,7 +1081,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="243">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1647,6 +1647,10 @@
     <xf numFmtId="0" fontId="80" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -19883,7 +19887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G52"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="101" min="1" max="1"/>
@@ -19912,7 +19916,7 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" s="101">
-      <c r="B4" s="127" t="inlineStr">
+      <c r="B4" s="194" t="inlineStr">
         <is>
           <t>Nome da Viagem</t>
         </is>
@@ -19925,548 +19929,561 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" s="101">
-      <c r="B5" s="130" t="inlineStr">
+      <c r="B5" s="194" t="inlineStr">
+        <is>
+          <t>🗺️ Cidade de Destino</t>
+        </is>
+      </c>
+      <c r="E5" s="243" t="inlineStr"/>
+      <c r="H5" s="244" t="inlineStr">
+        <is>
+          <t>← Ex: Florianópolis, SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="101">
+      <c r="B6" s="130" t="inlineStr">
         <is>
           <t>Data de Saída</t>
         </is>
       </c>
-      <c r="C5" s="128" t="n"/>
-      <c r="D5" s="131" t="inlineStr">
+      <c r="C6" s="128" t="n"/>
+      <c r="D6" s="131" t="inlineStr">
         <is>
           <t>← preencha a data de saída</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" s="101">
-      <c r="B6" s="127" t="inlineStr">
+    <row r="7" ht="22" customHeight="1" s="101">
+      <c r="B7" s="194" t="inlineStr">
         <is>
           <t>Data de Retorno</t>
         </is>
       </c>
-      <c r="C6" s="128" t="n"/>
-      <c r="D6" s="132">
+      <c r="C7" s="128" t="n"/>
+      <c r="D7" s="132">
         <f>IF(AND(C5&lt;&gt;"",C6&lt;&gt;""),TEXT(C6-C5,"0")&amp;" dias","— informe as datas")</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" s="101">
-      <c r="B7" s="130" t="inlineStr">
+    <row r="8" ht="22" customHeight="1" s="101">
+      <c r="B8" s="130" t="inlineStr">
         <is>
           <t>Nº de Pessoas</t>
         </is>
       </c>
-      <c r="C7" s="128" t="n">
+      <c r="C8" s="128" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="133" t="n"/>
-      <c r="E7" s="133" t="n"/>
-      <c r="F7" s="133" t="n"/>
-      <c r="G7" s="133" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1" s="101">
-      <c r="B8" s="127" t="inlineStr">
+      <c r="D8" s="133" t="n"/>
+      <c r="E8" s="133" t="n"/>
+      <c r="F8" s="133" t="n"/>
+      <c r="G8" s="133" t="n"/>
+    </row>
+    <row r="9" ht="10" customHeight="1" s="101">
+      <c r="B9" s="194" t="inlineStr">
         <is>
           <t>Orçamento Total (R$)</t>
         </is>
       </c>
-      <c r="C8" s="134" t="n">
+      <c r="C9" s="134" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="135" t="n"/>
-      <c r="E8" s="135" t="n"/>
-      <c r="F8" s="135" t="n"/>
-      <c r="G8" s="135" t="n"/>
-    </row>
-    <row r="9" ht="10" customHeight="1" s="101"/>
-    <row r="10" ht="26" customHeight="1" s="101">
-      <c r="B10" s="136" t="inlineStr">
+      <c r="D9" s="135" t="n"/>
+      <c r="E9" s="135" t="n"/>
+      <c r="F9" s="135" t="n"/>
+      <c r="G9" s="135" t="n"/>
+    </row>
+    <row r="10" ht="26" customHeight="1" s="101"/>
+    <row r="11" ht="22" customHeight="1" s="101">
+      <c r="B11" s="136" t="inlineStr">
         <is>
           <t>⛽  CALCULADORA DE COMBUSTÍVEL</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1" s="101">
-      <c r="B11" s="137" t="inlineStr">
+    <row r="12" ht="22" customHeight="1" s="101">
+      <c r="B12" s="229" t="inlineStr">
         <is>
           <t>Distância total (km)</t>
         </is>
       </c>
-      <c r="C11" s="138" t="n">
+      <c r="C12" s="138" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="133" t="n"/>
-      <c r="E11" s="131" t="inlineStr">
+      <c r="D12" s="133" t="n"/>
+      <c r="E12" s="131" t="inlineStr">
         <is>
           <t>Ida + volta. Ex: SP→Floripa = 600km × 2</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1" s="101">
-      <c r="B12" s="139" t="inlineStr">
+    <row r="13" ht="22" customHeight="1" s="101">
+      <c r="B13" s="139" t="inlineStr">
         <is>
           <t>Consumo do carro (km/L)</t>
         </is>
       </c>
-      <c r="C12" s="140" t="n">
+      <c r="C13" s="140" t="n">
         <v>12</v>
       </c>
-      <c r="D12" s="141" t="n"/>
-      <c r="E12" s="142" t="inlineStr">
+      <c r="D13" s="141" t="n"/>
+      <c r="E13" s="142" t="inlineStr">
         <is>
           <t>Consulte o manual do veículo</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1" s="101">
-      <c r="B13" s="137" t="inlineStr">
+    <row r="14" ht="22" customHeight="1" s="101">
+      <c r="B14" s="229" t="inlineStr">
         <is>
           <t>Tipo de combustível</t>
         </is>
       </c>
-      <c r="C13" s="143" t="inlineStr">
+      <c r="C14" s="143" t="inlineStr">
         <is>
           <t>Gasolina</t>
         </is>
       </c>
-      <c r="D13" s="133" t="n"/>
-      <c r="E13" s="131" t="inlineStr">
+      <c r="D14" s="133" t="n"/>
+      <c r="E14" s="131" t="inlineStr">
         <is>
           <t>Gasolina / Etanol / Diesel</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" s="101">
-      <c r="B14" s="139" t="inlineStr">
+    <row r="15" ht="22" customHeight="1" s="101">
+      <c r="B15" s="139" t="inlineStr">
         <is>
           <t>Preço do combustível (R$/L)</t>
         </is>
       </c>
-      <c r="C14" s="144" t="n">
+      <c r="C15" s="144" t="n">
         <v>5.5</v>
       </c>
-      <c r="D14" s="141" t="n"/>
-      <c r="E14" s="142" t="inlineStr">
+      <c r="D15" s="141" t="n"/>
+      <c r="E15" s="142" t="inlineStr">
         <is>
           <t>← insira o preço atual (veja nota abaixo)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1" s="101">
-      <c r="B15" s="145" t="inlineStr">
+    <row r="16" ht="22" customHeight="1" s="101">
+      <c r="B16" s="145" t="inlineStr">
         <is>
           <t>— Litros necessários</t>
         </is>
       </c>
-      <c r="C15" s="146">
+      <c r="C16" s="146">
         <f>IFERROR(C11/C12,0)</f>
         <v/>
       </c>
-      <c r="D15" s="133" t="n"/>
-      <c r="E15" s="131">
+      <c r="D16" s="133" t="n"/>
+      <c r="E16" s="131">
         <f> distância ÷ consumo</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1" s="101">
-      <c r="B16" s="147" t="inlineStr">
+    <row r="17" ht="22" customHeight="1" s="101">
+      <c r="B17" s="147" t="inlineStr">
         <is>
           <t>— Custo total combustível</t>
         </is>
       </c>
-      <c r="C16" s="148">
+      <c r="C17" s="148">
         <f>IFERROR(C15*C14,0)</f>
         <v/>
       </c>
-      <c r="D16" s="141" t="n"/>
-      <c r="E16" s="142">
+      <c r="D17" s="141" t="n"/>
+      <c r="E17" s="142">
         <f> litros × preço</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" s="101">
-      <c r="B17" s="145" t="inlineStr">
+    <row r="18" ht="28" customHeight="1" s="101">
+      <c r="B18" s="145" t="inlineStr">
         <is>
           <t>— Custo por pessoa</t>
         </is>
       </c>
-      <c r="C17" s="148">
+      <c r="C18" s="148">
         <f>IFERROR(C16/C7,0)</f>
         <v/>
       </c>
-      <c r="D17" s="133" t="n"/>
-      <c r="E17" s="131">
+      <c r="D18" s="133" t="n"/>
+      <c r="E18" s="131">
         <f> custo total ÷ nº pessoas (C7)</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1" s="101">
-      <c r="B18" s="149" t="inlineStr">
+    <row r="19" ht="10" customHeight="1" s="101">
+      <c r="B19" s="149" t="inlineStr">
         <is>
           <t>💡 Preço do combustível: consulte https://www.gov.br/anp (média semanal por estado) ou apps como Waze / Meu Combustível / Postos da Cidade.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="10" customHeight="1" s="101"/>
-    <row r="20" ht="26" customHeight="1" s="101">
-      <c r="B20" s="150" t="inlineStr">
+    <row r="20" ht="26" customHeight="1" s="101"/>
+    <row r="21" ht="20" customHeight="1" s="101">
+      <c r="B21" s="150" t="inlineStr">
         <is>
           <t>🏨  HOSPEDAGEM</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1" s="101">
-      <c r="B21" s="151" t="inlineStr">
+    <row r="22" ht="20" customHeight="1" s="101">
+      <c r="B22" s="213" t="inlineStr">
         <is>
           <t>Local / Acomodação</t>
         </is>
       </c>
-      <c r="C21" s="151" t="inlineStr">
+      <c r="C22" s="213" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="D21" s="151" t="inlineStr">
+      <c r="D22" s="213" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E21" s="151" t="inlineStr">
+      <c r="E22" s="213" t="inlineStr">
         <is>
           <t>Noites</t>
         </is>
       </c>
-      <c r="F21" s="151" t="inlineStr">
+      <c r="F22" s="213" t="inlineStr">
         <is>
           <t>R$/Noite</t>
         </is>
       </c>
-      <c r="G21" s="151" t="inlineStr">
+      <c r="G22" s="213" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1" s="101">
-      <c r="B22" s="152" t="n"/>
-      <c r="C22" s="152" t="n"/>
-      <c r="D22" s="152" t="n"/>
-      <c r="E22" s="153">
+    <row r="23" ht="20" customHeight="1" s="101">
+      <c r="B23" s="152" t="n"/>
+      <c r="C23" s="152" t="n"/>
+      <c r="D23" s="152" t="n"/>
+      <c r="E23" s="153">
         <f>IFERROR(D22-C22,0)</f>
         <v/>
       </c>
-      <c r="F22" s="154" t="n"/>
-      <c r="G22" s="155">
+      <c r="F23" s="154" t="n"/>
+      <c r="G23" s="155">
         <f>IFERROR(E22*F22,0)</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1" s="101">
-      <c r="B23" s="156" t="n"/>
-      <c r="C23" s="156" t="n"/>
-      <c r="D23" s="156" t="n"/>
-      <c r="E23" s="157">
+    <row r="24" ht="20" customHeight="1" s="101">
+      <c r="B24" s="156" t="n"/>
+      <c r="C24" s="156" t="n"/>
+      <c r="D24" s="156" t="n"/>
+      <c r="E24" s="157">
         <f>IFERROR(D23-C23,0)</f>
         <v/>
       </c>
-      <c r="F23" s="158" t="n"/>
-      <c r="G23" s="159">
+      <c r="F24" s="158" t="n"/>
+      <c r="G24" s="196">
         <f>IFERROR(E23*F23,0)</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1" s="101">
-      <c r="B24" s="152" t="n"/>
-      <c r="C24" s="152" t="n"/>
-      <c r="D24" s="152" t="n"/>
-      <c r="E24" s="153">
+    <row r="25" ht="20" customHeight="1" s="101">
+      <c r="B25" s="152" t="n"/>
+      <c r="C25" s="152" t="n"/>
+      <c r="D25" s="152" t="n"/>
+      <c r="E25" s="153">
         <f>IFERROR(D24-C24,0)</f>
         <v/>
       </c>
-      <c r="F24" s="154" t="n"/>
-      <c r="G24" s="155">
+      <c r="F25" s="154" t="n"/>
+      <c r="G25" s="155">
         <f>IFERROR(E24*F24,0)</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1" s="101">
-      <c r="B25" s="156" t="n"/>
-      <c r="C25" s="156" t="n"/>
-      <c r="D25" s="156" t="n"/>
-      <c r="E25" s="157">
+    <row r="26" ht="20" customHeight="1" s="101">
+      <c r="B26" s="156" t="n"/>
+      <c r="C26" s="156" t="n"/>
+      <c r="D26" s="156" t="n"/>
+      <c r="E26" s="157">
         <f>IFERROR(D25-C25,0)</f>
         <v/>
       </c>
-      <c r="F25" s="158" t="n"/>
-      <c r="G25" s="159">
+      <c r="F26" s="158" t="n"/>
+      <c r="G26" s="196">
         <f>IFERROR(E25*F25,0)</f>
         <v/>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1" s="101">
-      <c r="B26" s="152" t="n"/>
-      <c r="C26" s="152" t="n"/>
-      <c r="D26" s="152" t="n"/>
-      <c r="E26" s="153">
+    <row r="27" ht="22" customHeight="1" s="101">
+      <c r="B27" s="152" t="n"/>
+      <c r="C27" s="152" t="n"/>
+      <c r="D27" s="152" t="n"/>
+      <c r="E27" s="153">
         <f>IFERROR(D26-C26,0)</f>
         <v/>
       </c>
-      <c r="F26" s="154" t="n"/>
-      <c r="G26" s="155">
+      <c r="F27" s="154" t="n"/>
+      <c r="G27" s="155">
         <f>IFERROR(E26*F26,0)</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1" s="101">
-      <c r="B27" s="160" t="inlineStr">
+    <row r="28" ht="10" customHeight="1" s="101">
+      <c r="B28" s="160" t="inlineStr">
         <is>
           <t>TOTAL HOSPEDAGEM</t>
         </is>
       </c>
-      <c r="G27" s="161">
+      <c r="G28" s="161">
         <f>SUM(G22:G26)</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="10" customHeight="1" s="101"/>
-    <row r="29" ht="26" customHeight="1" s="101">
-      <c r="B29" s="162" t="inlineStr">
+    <row r="29" ht="26" customHeight="1" s="101"/>
+    <row r="30" ht="22" customHeight="1" s="101">
+      <c r="B30" s="162" t="inlineStr">
         <is>
           <t>🍽️  ALIMENTAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1" s="101">
-      <c r="B30" s="163" t="inlineStr">
+    <row r="31" ht="22" customHeight="1" s="101">
+      <c r="B31" s="197" t="inlineStr">
         <is>
           <t>Custo estimado por pessoa/dia (R$)</t>
         </is>
       </c>
-      <c r="C30" s="164" t="n">
+      <c r="C31" s="164" t="n">
         <v>80</v>
       </c>
-      <c r="D30" s="135" t="n"/>
-      <c r="E30" s="135" t="n"/>
-      <c r="F30" s="135" t="n"/>
-      <c r="G30" s="135" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1" s="101">
-      <c r="B31" s="137" t="inlineStr">
+      <c r="D31" s="135" t="n"/>
+      <c r="E31" s="135" t="n"/>
+      <c r="F31" s="135" t="n"/>
+      <c r="G31" s="135" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" s="101">
+      <c r="B32" s="229" t="inlineStr">
         <is>
           <t>Número de dias</t>
         </is>
       </c>
-      <c r="C31" s="165">
+      <c r="C32" s="165">
         <f>IFERROR(C6-C5,0)</f>
         <v/>
       </c>
-      <c r="D31" s="133" t="n"/>
-      <c r="E31" s="133" t="n"/>
-      <c r="F31" s="133" t="n"/>
-      <c r="G31" s="133" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1" s="101">
-      <c r="B32" s="163" t="inlineStr">
+      <c r="D32" s="133" t="n"/>
+      <c r="E32" s="133" t="n"/>
+      <c r="F32" s="133" t="n"/>
+      <c r="G32" s="133" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="101">
+      <c r="B33" s="197" t="inlineStr">
         <is>
           <t>Número de pessoas</t>
         </is>
       </c>
-      <c r="C32" s="166">
+      <c r="C33" s="166">
         <f>C7</f>
         <v/>
       </c>
-      <c r="D32" s="135" t="n"/>
-      <c r="E32" s="135" t="n"/>
-      <c r="F32" s="135" t="n"/>
-      <c r="G32" s="135" t="n"/>
-    </row>
-    <row r="33" ht="22" customHeight="1" s="101">
-      <c r="B33" s="167" t="inlineStr">
+      <c r="D33" s="135" t="n"/>
+      <c r="E33" s="135" t="n"/>
+      <c r="F33" s="135" t="n"/>
+      <c r="G33" s="135" t="n"/>
+    </row>
+    <row r="34" ht="10" customHeight="1" s="101">
+      <c r="B34" s="167" t="inlineStr">
         <is>
           <t>— TOTAL ALIMENTAÇÃO</t>
         </is>
       </c>
-      <c r="C33" s="168">
+      <c r="C34" s="168">
         <f>IFERROR(C30*C31*C32,0)</f>
         <v/>
       </c>
-      <c r="D33" s="169" t="n"/>
-      <c r="E33" s="169" t="n"/>
-      <c r="F33" s="169" t="n"/>
-      <c r="G33" s="169" t="n"/>
-    </row>
-    <row r="34" ht="10" customHeight="1" s="101"/>
-    <row r="35" ht="26" customHeight="1" s="101">
-      <c r="B35" s="170" t="inlineStr">
+      <c r="D34" s="169" t="n"/>
+      <c r="E34" s="169" t="n"/>
+      <c r="F34" s="169" t="n"/>
+      <c r="G34" s="169" t="n"/>
+    </row>
+    <row r="35" ht="26" customHeight="1" s="101"/>
+    <row r="36" ht="20" customHeight="1" s="101">
+      <c r="B36" s="170" t="inlineStr">
         <is>
           <t>🎡  PASSEIOS E OUTROS</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1" s="101">
-      <c r="B36" s="151" t="inlineStr">
+    <row r="37" ht="20" customHeight="1" s="101">
+      <c r="B37" s="213" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="C36" s="151" t="inlineStr">
+      <c r="C37" s="213" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D36" s="171" t="n"/>
-      <c r="E36" s="171" t="n"/>
-      <c r="F36" s="171" t="n"/>
-      <c r="G36" s="151" t="inlineStr">
+      <c r="D37" s="171" t="n"/>
+      <c r="E37" s="171" t="n"/>
+      <c r="F37" s="171" t="n"/>
+      <c r="G37" s="213" t="inlineStr">
         <is>
           <t>Valor (R$)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1" s="101">
-      <c r="B37" s="172" t="n"/>
-      <c r="C37" s="172" t="n"/>
-      <c r="D37" s="172" t="n"/>
-      <c r="E37" s="172" t="n"/>
-      <c r="F37" s="172" t="n"/>
-      <c r="G37" s="173" t="n"/>
-    </row>
     <row r="38" ht="20" customHeight="1" s="101">
-      <c r="B38" s="133" t="n"/>
-      <c r="C38" s="133" t="n"/>
-      <c r="D38" s="133" t="n"/>
-      <c r="E38" s="133" t="n"/>
-      <c r="F38" s="133" t="n"/>
-      <c r="G38" s="174" t="n"/>
+      <c r="B38" s="172" t="n"/>
+      <c r="C38" s="172" t="n"/>
+      <c r="D38" s="172" t="n"/>
+      <c r="E38" s="172" t="n"/>
+      <c r="F38" s="172" t="n"/>
+      <c r="G38" s="173" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1" s="101">
-      <c r="B39" s="172" t="n"/>
-      <c r="C39" s="172" t="n"/>
-      <c r="D39" s="172" t="n"/>
-      <c r="E39" s="172" t="n"/>
-      <c r="F39" s="172" t="n"/>
-      <c r="G39" s="173" t="n"/>
+      <c r="B39" s="133" t="n"/>
+      <c r="C39" s="133" t="n"/>
+      <c r="D39" s="133" t="n"/>
+      <c r="E39" s="133" t="n"/>
+      <c r="F39" s="133" t="n"/>
+      <c r="G39" s="221" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1" s="101">
-      <c r="B40" s="133" t="n"/>
-      <c r="C40" s="133" t="n"/>
-      <c r="D40" s="133" t="n"/>
-      <c r="E40" s="133" t="n"/>
-      <c r="F40" s="133" t="n"/>
-      <c r="G40" s="174" t="n"/>
+      <c r="B40" s="172" t="n"/>
+      <c r="C40" s="172" t="n"/>
+      <c r="D40" s="172" t="n"/>
+      <c r="E40" s="172" t="n"/>
+      <c r="F40" s="172" t="n"/>
+      <c r="G40" s="173" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1" s="101">
-      <c r="B41" s="172" t="n"/>
-      <c r="C41" s="172" t="n"/>
-      <c r="D41" s="172" t="n"/>
-      <c r="E41" s="172" t="n"/>
-      <c r="F41" s="172" t="n"/>
-      <c r="G41" s="173" t="n"/>
+      <c r="B41" s="133" t="n"/>
+      <c r="C41" s="133" t="n"/>
+      <c r="D41" s="133" t="n"/>
+      <c r="E41" s="133" t="n"/>
+      <c r="F41" s="133" t="n"/>
+      <c r="G41" s="221" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1" s="101">
-      <c r="B42" s="133" t="n"/>
-      <c r="C42" s="133" t="n"/>
-      <c r="D42" s="133" t="n"/>
-      <c r="E42" s="133" t="n"/>
-      <c r="F42" s="133" t="n"/>
-      <c r="G42" s="174" t="n"/>
+      <c r="B42" s="172" t="n"/>
+      <c r="C42" s="172" t="n"/>
+      <c r="D42" s="172" t="n"/>
+      <c r="E42" s="172" t="n"/>
+      <c r="F42" s="172" t="n"/>
+      <c r="G42" s="173" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1" s="101">
-      <c r="B43" s="175" t="inlineStr">
+      <c r="B43" s="133" t="n"/>
+      <c r="C43" s="133" t="n"/>
+      <c r="D43" s="133" t="n"/>
+      <c r="E43" s="133" t="n"/>
+      <c r="F43" s="133" t="n"/>
+      <c r="G43" s="221" t="n"/>
+    </row>
+    <row r="44" ht="10" customHeight="1" s="101">
+      <c r="B44" s="175" t="inlineStr">
         <is>
           <t>TOTAL OUTROS</t>
         </is>
       </c>
-      <c r="G43" s="176">
+      <c r="G44" s="176">
         <f>SUM(G37:G42)</f>
         <v/>
       </c>
     </row>
-    <row r="44" ht="10" customHeight="1" s="101"/>
-    <row r="45" ht="26" customHeight="1" s="101">
-      <c r="B45" s="177" t="inlineStr">
+    <row r="45" ht="26" customHeight="1" s="101"/>
+    <row r="46" ht="22" customHeight="1" s="101">
+      <c r="B46" s="177" t="inlineStr">
         <is>
           <t>💰  RESUMO TOTAL DA VIAGEM</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1" s="101">
-      <c r="B46" s="178" t="inlineStr">
+    <row r="47" ht="22" customHeight="1" s="101">
+      <c r="B47" s="178" t="inlineStr">
         <is>
           <t>⛽ Combustível</t>
         </is>
       </c>
-      <c r="G46" s="179">
+      <c r="G47" s="179">
         <f>C16</f>
         <v/>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1" s="101">
-      <c r="B47" s="180" t="inlineStr">
+    <row r="48" ht="22" customHeight="1" s="101">
+      <c r="B48" s="180" t="inlineStr">
         <is>
           <t>🏨 Hospedagem</t>
         </is>
       </c>
-      <c r="G47" s="181">
+      <c r="G48" s="181">
         <f>G27</f>
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1" s="101">
-      <c r="B48" s="182" t="inlineStr">
+    <row r="49" ht="22" customHeight="1" s="101">
+      <c r="B49" s="182" t="inlineStr">
         <is>
           <t>🍽️ Alimentação</t>
         </is>
       </c>
-      <c r="G48" s="183">
+      <c r="G49" s="235">
         <f>C33</f>
         <v/>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1" s="101">
-      <c r="B49" s="184" t="inlineStr">
+    <row r="50" ht="36" customHeight="1" s="101">
+      <c r="B50" s="184" t="inlineStr">
         <is>
           <t>🎡 Outros</t>
         </is>
       </c>
-      <c r="G49" s="185">
+      <c r="G50" s="185">
         <f>G43</f>
         <v/>
       </c>
     </row>
-    <row r="50" ht="36" customHeight="1" s="101">
-      <c r="B50" s="186" t="inlineStr">
+    <row r="51" ht="22" customHeight="1" s="101">
+      <c r="B51" s="186" t="inlineStr">
         <is>
           <t>🧳 TOTAL DA VIAGEM</t>
         </is>
       </c>
-      <c r="G50" s="187">
+      <c r="G51" s="187">
         <f>SUM(G46:G49)</f>
         <v/>
       </c>
     </row>
-    <row r="51" ht="22" customHeight="1" s="101">
-      <c r="B51" s="188" t="inlineStr">
+    <row r="52" ht="22" customHeight="1" s="101">
+      <c r="B52" s="188" t="inlineStr">
         <is>
           <t>👤 Total por pessoa</t>
         </is>
       </c>
-      <c r="G51" s="189">
+      <c r="G52" s="189">
         <f>IFERROR(G50/C7,0)</f>
         <v/>
       </c>
     </row>
-    <row r="52" ht="22" customHeight="1" s="101">
-      <c r="B52" s="190">
+    <row r="53">
+      <c r="B53" s="190">
         <f>IF(C8-G50&gt;=0,"✅ Sobra do orçamento","⚠️ Estouro do orçamento")</f>
         <v/>
       </c>
-      <c r="G52" s="191">
+      <c r="G53" s="191">
         <f>C8-G50</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B1:G1"/>
@@ -20482,6 +20499,7 @@
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B5:D5"/>
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="B45:G45"/>
     <mergeCell ref="B35:G35"/>

</xml_diff>

<commit_message>
chore: regenerar planilha completa (todas as abas) e corrigir menu do script
</commit_message>
<xml_diff>
--- a/controle-financeiro-final.xlsx
+++ b/controle-financeiro-final.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="dd/MM/yyyy"/>
@@ -29,13 +29,14 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="dd/MM/yyyy HH:mm"/>
     <numFmt numFmtId="170" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="171" formatCode="0.0"/>
-    <numFmt numFmtId="172" formatCode="0 &quot;meses&quot;"/>
-    <numFmt numFmtId="173" formatCode="MMM/YYYY"/>
-    <numFmt numFmtId="174" formatCode="0&quot;%&quot;"/>
-    <numFmt numFmtId="175" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="171" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="172" formatCode="0 &quot;dias&quot;"/>
+    <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="0 &quot;meses&quot;"/>
+    <numFmt numFmtId="175" formatCode="MMM/YYYY"/>
+    <numFmt numFmtId="176" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="81">
+  <fonts count="78">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -305,24 +306,6 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00AAAAAA"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0016A085"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <color rgb="001B2A4A"/>
       <sz val="10"/>
     </font>
@@ -330,6 +313,12 @@
       <name val="Segoe UI"/>
       <color rgb="002980B9"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -342,12 +331,6 @@
       <b val="1"/>
       <color rgb="00E67E22"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00E67E22"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -439,6 +422,7 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="001A5276"/>
       <sz val="10"/>
     </font>
@@ -463,12 +447,6 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001A5276"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="0016A085"/>
       <sz val="14"/>
     </font>
@@ -486,13 +464,18 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00AAAAAA"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <color rgb="00E74C3C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="0016A085"/>
       <sz val="9"/>
     </font>
     <font>
@@ -530,7 +513,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill/>
     </fill>
@@ -612,6 +595,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFBFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1081,7 +1069,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="245">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1319,338 +1307,293 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="41" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="41" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="41" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="43" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="44" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="43" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="43" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="43" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="46" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="46" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="48" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="48" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="49" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="50" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="50" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="50" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="52" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="53" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="54" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="46" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="48" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="48" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="52" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="53" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="58" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="59" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="60" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="37" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="45" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="51" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="50" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="52" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="57" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="53" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="53" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="53" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="55" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="45" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="57" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="48" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="41" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="61" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="62" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="37" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="64" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="61" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="63" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="51" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="60" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="60" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="64" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="65" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="66" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="66" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="68" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="62" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="70" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="71" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="73" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="70" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="71" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="73" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="74" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="65" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="75" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="52" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="75" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="66" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="63" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="63" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="63" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="67" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="68" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="70" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="70" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="72" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="69" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="73" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="45" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="74" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="44" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="75" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="76" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="73" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="74" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="44" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="75" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="76" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="78" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="77" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="55" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="78" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="66" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="66" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="79" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="76" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="80" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="77" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3590,11 +3533,11 @@
     <row r="1000" ht="15.75" customHeight="1" s="101"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="J3:K3"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="D3:G3"/>
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="J3:K3"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="A19:K19"/>
@@ -4291,7 +4234,7 @@
       </c>
       <c r="H18" s="77" t="inlineStr">
         <is>
-          <t>A Pagar</t>
+          <t>A Receber</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4270,7 @@
       </c>
       <c r="H19" s="77" t="inlineStr">
         <is>
-          <t>A Pagar</t>
+          <t>A Receber</t>
         </is>
       </c>
     </row>
@@ -19887,7 +19830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="101" min="1" max="1"/>
@@ -19901,626 +19844,827 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" s="101">
-      <c r="B1" s="125" t="inlineStr">
-        <is>
-          <t>✈️  PLANEJAMENTO DE VIAGEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="8" customHeight="1" s="101"/>
+      <c r="A1" s="125" t="n"/>
+      <c r="B1" s="126" t="inlineStr">
+        <is>
+          <t>PLANEJAMENTO DE VIAGEM</t>
+        </is>
+      </c>
+      <c r="H1" s="125" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="125" t="n"/>
+      <c r="B2" s="125" t="n"/>
+      <c r="C2" s="125" t="n"/>
+      <c r="D2" s="125" t="n"/>
+      <c r="E2" s="125" t="n"/>
+      <c r="F2" s="125" t="n"/>
+      <c r="G2" s="125" t="n"/>
+      <c r="H2" s="125" t="n"/>
+    </row>
     <row r="3" ht="26" customHeight="1" s="101">
-      <c r="B3" s="126" t="inlineStr">
-        <is>
-          <t>📋  DADOS DA VIAGEM</t>
-        </is>
-      </c>
+      <c r="A3" s="125" t="n"/>
+      <c r="B3" s="127" t="inlineStr">
+        <is>
+          <t>DADOS DA VIAGEM</t>
+        </is>
+      </c>
+      <c r="H3" s="125" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1" s="101">
-      <c r="B4" s="194" t="inlineStr">
+      <c r="A4" s="125" t="n"/>
+      <c r="B4" s="128" t="inlineStr">
         <is>
           <t>Nome da Viagem</t>
         </is>
       </c>
-      <c r="C4" s="128" t="inlineStr"/>
-      <c r="D4" s="129" t="inlineStr">
-        <is>
-          <t>Ex: Viagem a Floripa</t>
-        </is>
-      </c>
+      <c r="C4" s="129" t="n"/>
+      <c r="F4" s="130" t="n"/>
+      <c r="G4" s="130" t="n"/>
+      <c r="H4" s="125" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1" s="101">
-      <c r="B5" s="194" t="inlineStr">
-        <is>
-          <t>🗺️ Cidade de Destino</t>
-        </is>
-      </c>
-      <c r="E5" s="243" t="inlineStr"/>
-      <c r="H5" s="244" t="inlineStr">
-        <is>
-          <t>← Ex: Florianópolis, SC</t>
-        </is>
-      </c>
+      <c r="A5" s="125" t="n"/>
+      <c r="B5" s="131" t="inlineStr">
+        <is>
+          <t>Cidade de Destino</t>
+        </is>
+      </c>
+      <c r="C5" s="129" t="inlineStr">
+        <is>
+          <t>Ex: Florianopolis, SC</t>
+        </is>
+      </c>
+      <c r="F5" s="132" t="n"/>
+      <c r="G5" s="132" t="n"/>
+      <c r="H5" s="125" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1" s="101">
-      <c r="B6" s="130" t="inlineStr">
-        <is>
-          <t>Data de Saída</t>
-        </is>
-      </c>
-      <c r="C6" s="128" t="n"/>
-      <c r="D6" s="131" t="inlineStr">
-        <is>
-          <t>← preencha a data de saída</t>
-        </is>
-      </c>
+      <c r="A6" s="125" t="n"/>
+      <c r="B6" s="128" t="inlineStr">
+        <is>
+          <t>Data de Saida</t>
+        </is>
+      </c>
+      <c r="C6" s="133" t="inlineStr">
+        <is>
+          <t>DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="D6" s="130" t="n"/>
+      <c r="E6" s="130" t="n"/>
+      <c r="F6" s="130" t="n"/>
+      <c r="G6" s="130" t="n"/>
+      <c r="H6" s="125" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1" s="101">
-      <c r="B7" s="194" t="inlineStr">
+      <c r="A7" s="125" t="n"/>
+      <c r="B7" s="131" t="inlineStr">
         <is>
           <t>Data de Retorno</t>
         </is>
       </c>
-      <c r="C7" s="128" t="n"/>
-      <c r="D7" s="132">
-        <f>IF(AND(C5&lt;&gt;"",C6&lt;&gt;""),TEXT(C6-C5,"0")&amp;" dias","— informe as datas")</f>
+      <c r="C7" s="133" t="n"/>
+      <c r="D7" s="132" t="n"/>
+      <c r="E7" s="132" t="n"/>
+      <c r="F7" s="132" t="n"/>
+      <c r="G7" s="132" t="n"/>
+      <c r="H7" s="125" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1" s="101">
+      <c r="A8" s="125" t="n"/>
+      <c r="B8" s="128" t="inlineStr">
+        <is>
+          <t>Dias de viagem</t>
+        </is>
+      </c>
+      <c r="C8" s="134">
+        <f>IFERROR(C7-C6,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" s="101">
-      <c r="B8" s="130" t="inlineStr">
-        <is>
-          <t>Nº de Pessoas</t>
-        </is>
-      </c>
-      <c r="C8" s="128" t="n">
+      <c r="D8" s="130" t="n"/>
+      <c r="E8" s="130" t="n"/>
+      <c r="F8" s="130" t="n"/>
+      <c r="G8" s="130" t="n"/>
+      <c r="H8" s="125" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" s="101">
+      <c r="A9" s="125" t="n"/>
+      <c r="B9" s="131" t="inlineStr">
+        <is>
+          <t>No de Pessoas</t>
+        </is>
+      </c>
+      <c r="C9" s="129" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="133" t="n"/>
-      <c r="E8" s="133" t="n"/>
-      <c r="F8" s="133" t="n"/>
-      <c r="G8" s="133" t="n"/>
-    </row>
-    <row r="9" ht="10" customHeight="1" s="101">
-      <c r="B9" s="194" t="inlineStr">
-        <is>
-          <t>Orçamento Total (R$)</t>
-        </is>
-      </c>
-      <c r="C9" s="134" t="n">
+      <c r="D9" s="132" t="n"/>
+      <c r="E9" s="132" t="n"/>
+      <c r="F9" s="132" t="n"/>
+      <c r="G9" s="132" t="n"/>
+      <c r="H9" s="125" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="101">
+      <c r="A10" s="125" t="n"/>
+      <c r="B10" s="128" t="inlineStr">
+        <is>
+          <t>Orcamento Total (R$)</t>
+        </is>
+      </c>
+      <c r="C10" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="135" t="n"/>
-      <c r="E9" s="135" t="n"/>
-      <c r="F9" s="135" t="n"/>
-      <c r="G9" s="135" t="n"/>
-    </row>
-    <row r="10" ht="26" customHeight="1" s="101"/>
-    <row r="11" ht="22" customHeight="1" s="101">
-      <c r="B11" s="136" t="inlineStr">
-        <is>
-          <t>⛽  CALCULADORA DE COMBUSTÍVEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" s="101">
-      <c r="B12" s="229" t="inlineStr">
-        <is>
-          <t>Distância total (km)</t>
-        </is>
-      </c>
-      <c r="C12" s="138" t="n">
+      <c r="D10" s="130" t="n"/>
+      <c r="E10" s="130" t="n"/>
+      <c r="F10" s="130" t="n"/>
+      <c r="G10" s="130" t="n"/>
+      <c r="H10" s="125" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="125" t="n"/>
+      <c r="B11" s="125" t="n"/>
+      <c r="C11" s="125" t="n"/>
+      <c r="D11" s="125" t="n"/>
+      <c r="E11" s="125" t="n"/>
+      <c r="F11" s="125" t="n"/>
+      <c r="G11" s="125" t="n"/>
+      <c r="H11" s="125" t="n"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" s="101">
+      <c r="A12" s="125" t="n"/>
+      <c r="B12" s="136" t="inlineStr">
+        <is>
+          <t>CALCULADORA DE COMBUSTIVEL</t>
+        </is>
+      </c>
+      <c r="H12" s="125" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="101">
+      <c r="A13" s="125" t="n"/>
+      <c r="B13" s="137" t="inlineStr">
+        <is>
+          <t>Distancia total (km)</t>
+        </is>
+      </c>
+      <c r="C13" s="138" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="133" t="n"/>
-      <c r="E12" s="131" t="inlineStr">
-        <is>
-          <t>Ida + volta. Ex: SP→Floripa = 600km × 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" s="101">
-      <c r="B13" s="139" t="inlineStr">
+      <c r="D13" s="132" t="n"/>
+      <c r="E13" s="139" t="inlineStr">
+        <is>
+          <t>Ida + volta</t>
+        </is>
+      </c>
+      <c r="H13" s="125" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="101">
+      <c r="A14" s="125" t="n"/>
+      <c r="B14" s="140" t="inlineStr">
         <is>
           <t>Consumo do carro (km/L)</t>
         </is>
       </c>
-      <c r="C13" s="140" t="n">
+      <c r="C14" s="141" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="141" t="n"/>
-      <c r="E13" s="142" t="inlineStr">
-        <is>
-          <t>Consulte o manual do veículo</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" s="101">
-      <c r="B14" s="229" t="inlineStr">
-        <is>
-          <t>Tipo de combustível</t>
-        </is>
-      </c>
-      <c r="C14" s="143" t="inlineStr">
-        <is>
-          <t>Gasolina</t>
-        </is>
-      </c>
-      <c r="D14" s="133" t="n"/>
-      <c r="E14" s="131" t="inlineStr">
-        <is>
-          <t>Gasolina / Etanol / Diesel</t>
-        </is>
-      </c>
+      <c r="D14" s="142" t="n"/>
+      <c r="E14" s="143" t="inlineStr">
+        <is>
+          <t>Verifique o manual do veiculo</t>
+        </is>
+      </c>
+      <c r="H14" s="125" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1" s="101">
-      <c r="B15" s="139" t="inlineStr">
-        <is>
-          <t>Preço do combustível (R$/L)</t>
+      <c r="A15" s="125" t="n"/>
+      <c r="B15" s="137" t="inlineStr">
+        <is>
+          <t>Preco do combustivel (R$/L)</t>
         </is>
       </c>
       <c r="C15" s="144" t="n">
         <v>5.5</v>
       </c>
-      <c r="D15" s="141" t="n"/>
-      <c r="E15" s="142" t="inlineStr">
-        <is>
-          <t>← insira o preço atual (veja nota abaixo)</t>
-        </is>
-      </c>
+      <c r="D15" s="132" t="n"/>
+      <c r="E15" s="139" t="inlineStr">
+        <is>
+          <t>Consulte gov.br/anp ou apps como Waze</t>
+        </is>
+      </c>
+      <c r="H15" s="125" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1" s="101">
+      <c r="A16" s="125" t="n"/>
       <c r="B16" s="145" t="inlineStr">
         <is>
-          <t>— Litros necessários</t>
+          <t>Litros necessarios</t>
         </is>
       </c>
       <c r="C16" s="146">
-        <f>IFERROR(C11/C12,0)</f>
+        <f>IFERROR(C13/C14,0)</f>
         <v/>
       </c>
-      <c r="D16" s="133" t="n"/>
-      <c r="E16" s="131">
-        <f> distância ÷ consumo</f>
+      <c r="D16" s="142" t="n"/>
+      <c r="E16" s="143">
+        <f> distancia / consumo</f>
         <v/>
       </c>
+      <c r="H16" s="125" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1" s="101">
+      <c r="A17" s="125" t="n"/>
       <c r="B17" s="147" t="inlineStr">
         <is>
-          <t>— Custo total combustível</t>
+          <t>Custo total combustivel</t>
         </is>
       </c>
       <c r="C17" s="148">
-        <f>IFERROR(C15*C14,0)</f>
+        <f>IFERROR(C16*C15,0)</f>
         <v/>
       </c>
-      <c r="D17" s="141" t="n"/>
-      <c r="E17" s="142">
-        <f> litros × preço</f>
+      <c r="D17" s="132" t="n"/>
+      <c r="E17" s="139">
+        <f> litros x preco</f>
         <v/>
       </c>
-    </row>
-    <row r="18" ht="28" customHeight="1" s="101">
+      <c r="H17" s="125" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1" s="101">
+      <c r="A18" s="125" t="n"/>
       <c r="B18" s="145" t="inlineStr">
         <is>
-          <t>— Custo por pessoa</t>
+          <t>Custo por pessoa</t>
         </is>
       </c>
       <c r="C18" s="148">
-        <f>IFERROR(C16/C7,0)</f>
+        <f>IFERROR(C17/C9,0)</f>
         <v/>
       </c>
-      <c r="D18" s="133" t="n"/>
-      <c r="E18" s="131">
-        <f> custo total ÷ nº pessoas (C7)</f>
+      <c r="D18" s="142" t="n"/>
+      <c r="E18" s="143">
+        <f> total / no pessoas</f>
         <v/>
       </c>
-    </row>
-    <row r="19" ht="10" customHeight="1" s="101">
-      <c r="B19" s="149" t="inlineStr">
-        <is>
-          <t>💡 Preço do combustível: consulte https://www.gov.br/anp (média semanal por estado) ou apps como Waze / Meu Combustível / Postos da Cidade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1" s="101"/>
+      <c r="H18" s="125" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="125" t="n"/>
+      <c r="B19" s="125" t="n"/>
+      <c r="C19" s="125" t="n"/>
+      <c r="D19" s="125" t="n"/>
+      <c r="E19" s="125" t="n"/>
+      <c r="F19" s="125" t="n"/>
+      <c r="G19" s="125" t="n"/>
+      <c r="H19" s="125" t="n"/>
+    </row>
+    <row r="20" ht="26" customHeight="1" s="101">
+      <c r="A20" s="125" t="n"/>
+      <c r="B20" s="149" t="inlineStr">
+        <is>
+          <t>HOSPEDAGEM</t>
+        </is>
+      </c>
+      <c r="H20" s="125" t="n"/>
+    </row>
     <row r="21" ht="20" customHeight="1" s="101">
+      <c r="A21" s="125" t="n"/>
       <c r="B21" s="150" t="inlineStr">
         <is>
-          <t>🏨  HOSPEDAGEM</t>
-        </is>
-      </c>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="C21" s="150" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="D21" s="150" t="inlineStr">
+        <is>
+          <t>Saida</t>
+        </is>
+      </c>
+      <c r="E21" s="150" t="inlineStr">
+        <is>
+          <t>Noites</t>
+        </is>
+      </c>
+      <c r="F21" s="150" t="inlineStr">
+        <is>
+          <t>R$/Noite</t>
+        </is>
+      </c>
+      <c r="G21" s="150" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H21" s="125" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1" s="101">
-      <c r="B22" s="213" t="inlineStr">
-        <is>
-          <t>Local / Acomodação</t>
-        </is>
-      </c>
-      <c r="C22" s="213" t="inlineStr">
-        <is>
-          <t>Entrada</t>
-        </is>
-      </c>
-      <c r="D22" s="213" t="inlineStr">
-        <is>
-          <t>Saída</t>
-        </is>
-      </c>
-      <c r="E22" s="213" t="inlineStr">
-        <is>
-          <t>Noites</t>
-        </is>
-      </c>
-      <c r="F22" s="213" t="inlineStr">
-        <is>
-          <t>R$/Noite</t>
-        </is>
-      </c>
-      <c r="G22" s="213" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1" s="101">
-      <c r="B23" s="152" t="n"/>
-      <c r="C23" s="152" t="n"/>
-      <c r="D23" s="152" t="n"/>
-      <c r="E23" s="153">
+      <c r="A22" s="125" t="n"/>
+      <c r="B22" s="130" t="n"/>
+      <c r="C22" s="130" t="n"/>
+      <c r="D22" s="130" t="n"/>
+      <c r="E22" s="151">
         <f>IFERROR(D22-C22,0)</f>
         <v/>
       </c>
-      <c r="F23" s="154" t="n"/>
-      <c r="G23" s="155">
+      <c r="F22" s="152" t="n"/>
+      <c r="G22" s="153">
         <f>IFERROR(E22*F22,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="24" ht="20" customHeight="1" s="101">
-      <c r="B24" s="156" t="n"/>
-      <c r="C24" s="156" t="n"/>
-      <c r="D24" s="156" t="n"/>
-      <c r="E24" s="157">
+      <c r="H22" s="125" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" s="101">
+      <c r="A23" s="125" t="n"/>
+      <c r="B23" s="132" t="n"/>
+      <c r="C23" s="132" t="n"/>
+      <c r="D23" s="132" t="n"/>
+      <c r="E23" s="154">
         <f>IFERROR(D23-C23,0)</f>
         <v/>
       </c>
-      <c r="F24" s="158" t="n"/>
-      <c r="G24" s="196">
+      <c r="F23" s="155" t="n"/>
+      <c r="G23" s="156">
         <f>IFERROR(E23*F23,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="25" ht="20" customHeight="1" s="101">
-      <c r="B25" s="152" t="n"/>
-      <c r="C25" s="152" t="n"/>
-      <c r="D25" s="152" t="n"/>
-      <c r="E25" s="153">
+      <c r="H23" s="125" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" s="101">
+      <c r="A24" s="125" t="n"/>
+      <c r="B24" s="130" t="n"/>
+      <c r="C24" s="130" t="n"/>
+      <c r="D24" s="130" t="n"/>
+      <c r="E24" s="151">
         <f>IFERROR(D24-C24,0)</f>
         <v/>
       </c>
-      <c r="F25" s="154" t="n"/>
-      <c r="G25" s="155">
+      <c r="F24" s="152" t="n"/>
+      <c r="G24" s="153">
         <f>IFERROR(E24*F24,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" s="101">
-      <c r="B26" s="156" t="n"/>
-      <c r="C26" s="156" t="n"/>
-      <c r="D26" s="156" t="n"/>
-      <c r="E26" s="157">
+      <c r="H24" s="125" t="n"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" s="101">
+      <c r="A25" s="125" t="n"/>
+      <c r="B25" s="132" t="n"/>
+      <c r="C25" s="132" t="n"/>
+      <c r="D25" s="132" t="n"/>
+      <c r="E25" s="154">
         <f>IFERROR(D25-C25,0)</f>
         <v/>
       </c>
-      <c r="F26" s="158" t="n"/>
-      <c r="G26" s="196">
+      <c r="F25" s="155" t="n"/>
+      <c r="G25" s="156">
         <f>IFERROR(E25*F25,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="27" ht="22" customHeight="1" s="101">
-      <c r="B27" s="152" t="n"/>
-      <c r="C27" s="152" t="n"/>
-      <c r="D27" s="152" t="n"/>
-      <c r="E27" s="153">
+      <c r="H25" s="125" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" s="101">
+      <c r="A26" s="125" t="n"/>
+      <c r="B26" s="130" t="n"/>
+      <c r="C26" s="130" t="n"/>
+      <c r="D26" s="130" t="n"/>
+      <c r="E26" s="151">
         <f>IFERROR(D26-C26,0)</f>
         <v/>
       </c>
-      <c r="F27" s="154" t="n"/>
-      <c r="G27" s="155">
+      <c r="F26" s="152" t="n"/>
+      <c r="G26" s="153">
         <f>IFERROR(E26*F26,0)</f>
         <v/>
       </c>
-    </row>
-    <row r="28" ht="10" customHeight="1" s="101">
-      <c r="B28" s="160" t="inlineStr">
+      <c r="H26" s="125" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" s="101">
+      <c r="A27" s="125" t="n"/>
+      <c r="B27" s="157" t="inlineStr">
         <is>
           <t>TOTAL HOSPEDAGEM</t>
         </is>
       </c>
-      <c r="G28" s="161">
+      <c r="G27" s="158">
         <f>SUM(G22:G26)</f>
         <v/>
       </c>
-    </row>
-    <row r="29" ht="26" customHeight="1" s="101"/>
+      <c r="H27" s="125" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="125" t="n"/>
+      <c r="B28" s="125" t="n"/>
+      <c r="C28" s="125" t="n"/>
+      <c r="D28" s="125" t="n"/>
+      <c r="E28" s="125" t="n"/>
+      <c r="F28" s="125" t="n"/>
+      <c r="G28" s="125" t="n"/>
+      <c r="H28" s="125" t="n"/>
+    </row>
+    <row r="29" ht="26" customHeight="1" s="101">
+      <c r="A29" s="125" t="n"/>
+      <c r="B29" s="159" t="inlineStr">
+        <is>
+          <t>ALIMENTACAO</t>
+        </is>
+      </c>
+      <c r="H29" s="125" t="n"/>
+    </row>
     <row r="30" ht="22" customHeight="1" s="101">
-      <c r="B30" s="162" t="inlineStr">
-        <is>
-          <t>🍽️  ALIMENTAÇÃO</t>
-        </is>
-      </c>
+      <c r="A30" s="125" t="n"/>
+      <c r="B30" s="160" t="inlineStr">
+        <is>
+          <t>Custo por pessoa/dia (R$)</t>
+        </is>
+      </c>
+      <c r="C30" s="161" t="n">
+        <v>80</v>
+      </c>
+      <c r="D30" s="130" t="n"/>
+      <c r="E30" s="130" t="n"/>
+      <c r="F30" s="130" t="n"/>
+      <c r="G30" s="130" t="n"/>
+      <c r="H30" s="125" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1" s="101">
-      <c r="B31" s="197" t="inlineStr">
-        <is>
-          <t>Custo estimado por pessoa/dia (R$)</t>
-        </is>
-      </c>
-      <c r="C31" s="164" t="n">
-        <v>80</v>
-      </c>
-      <c r="D31" s="135" t="n"/>
-      <c r="E31" s="135" t="n"/>
-      <c r="F31" s="135" t="n"/>
-      <c r="G31" s="135" t="n"/>
+      <c r="A31" s="125" t="n"/>
+      <c r="B31" s="137" t="inlineStr">
+        <is>
+          <t>Numero de dias</t>
+        </is>
+      </c>
+      <c r="C31" s="162">
+        <f>IFERROR(C8,0)</f>
+        <v/>
+      </c>
+      <c r="D31" s="132" t="n"/>
+      <c r="E31" s="132" t="n"/>
+      <c r="F31" s="132" t="n"/>
+      <c r="G31" s="132" t="n"/>
+      <c r="H31" s="125" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1" s="101">
-      <c r="B32" s="229" t="inlineStr">
-        <is>
-          <t>Número de dias</t>
-        </is>
-      </c>
-      <c r="C32" s="165">
-        <f>IFERROR(C6-C5,0)</f>
+      <c r="A32" s="125" t="n"/>
+      <c r="B32" s="160" t="inlineStr">
+        <is>
+          <t>Numero de pessoas</t>
+        </is>
+      </c>
+      <c r="C32" s="163">
+        <f>C9</f>
         <v/>
       </c>
-      <c r="D32" s="133" t="n"/>
-      <c r="E32" s="133" t="n"/>
-      <c r="F32" s="133" t="n"/>
-      <c r="G32" s="133" t="n"/>
+      <c r="D32" s="130" t="n"/>
+      <c r="E32" s="130" t="n"/>
+      <c r="F32" s="130" t="n"/>
+      <c r="G32" s="130" t="n"/>
+      <c r="H32" s="125" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1" s="101">
-      <c r="B33" s="197" t="inlineStr">
-        <is>
-          <t>Número de pessoas</t>
-        </is>
-      </c>
-      <c r="C33" s="166">
-        <f>C7</f>
-        <v/>
-      </c>
-      <c r="D33" s="135" t="n"/>
-      <c r="E33" s="135" t="n"/>
-      <c r="F33" s="135" t="n"/>
-      <c r="G33" s="135" t="n"/>
-    </row>
-    <row r="34" ht="10" customHeight="1" s="101">
-      <c r="B34" s="167" t="inlineStr">
-        <is>
-          <t>— TOTAL ALIMENTAÇÃO</t>
-        </is>
-      </c>
-      <c r="C34" s="168">
+      <c r="A33" s="125" t="n"/>
+      <c r="B33" s="164" t="inlineStr">
+        <is>
+          <t>TOTAL ALIMENTACAO</t>
+        </is>
+      </c>
+      <c r="C33" s="165">
         <f>IFERROR(C30*C31*C32,0)</f>
         <v/>
       </c>
-      <c r="D34" s="169" t="n"/>
-      <c r="E34" s="169" t="n"/>
-      <c r="F34" s="169" t="n"/>
-      <c r="G34" s="169" t="n"/>
-    </row>
-    <row r="35" ht="26" customHeight="1" s="101"/>
+      <c r="D33" s="166" t="n"/>
+      <c r="E33" s="166" t="n"/>
+      <c r="F33" s="166" t="n"/>
+      <c r="G33" s="166" t="n"/>
+      <c r="H33" s="125" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="125" t="n"/>
+      <c r="B34" s="125" t="n"/>
+      <c r="C34" s="125" t="n"/>
+      <c r="D34" s="125" t="n"/>
+      <c r="E34" s="125" t="n"/>
+      <c r="F34" s="125" t="n"/>
+      <c r="G34" s="125" t="n"/>
+      <c r="H34" s="125" t="n"/>
+    </row>
+    <row r="35" ht="26" customHeight="1" s="101">
+      <c r="A35" s="125" t="n"/>
+      <c r="B35" s="167" t="inlineStr">
+        <is>
+          <t>PASSEIOS E OUTROS</t>
+        </is>
+      </c>
+      <c r="H35" s="125" t="n"/>
+    </row>
     <row r="36" ht="20" customHeight="1" s="101">
-      <c r="B36" s="170" t="inlineStr">
-        <is>
-          <t>🎡  PASSEIOS E OUTROS</t>
-        </is>
-      </c>
+      <c r="A36" s="125" t="n"/>
+      <c r="B36" s="168" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+      <c r="C36" s="169" t="n"/>
+      <c r="D36" s="169" t="n"/>
+      <c r="E36" s="169" t="n"/>
+      <c r="F36" s="169" t="n"/>
+      <c r="G36" s="150" t="inlineStr">
+        <is>
+          <t>Valor (R$)</t>
+        </is>
+      </c>
+      <c r="H36" s="125" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1" s="101">
-      <c r="B37" s="213" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
-      <c r="C37" s="213" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D37" s="171" t="n"/>
-      <c r="E37" s="171" t="n"/>
-      <c r="F37" s="171" t="n"/>
-      <c r="G37" s="213" t="inlineStr">
-        <is>
-          <t>Valor (R$)</t>
-        </is>
-      </c>
+      <c r="A37" s="125" t="n"/>
+      <c r="B37" s="170" t="n"/>
+      <c r="C37" s="170" t="n"/>
+      <c r="D37" s="170" t="n"/>
+      <c r="E37" s="170" t="n"/>
+      <c r="F37" s="170" t="n"/>
+      <c r="G37" s="171" t="n"/>
+      <c r="H37" s="125" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1" s="101">
-      <c r="B38" s="172" t="n"/>
-      <c r="C38" s="172" t="n"/>
-      <c r="D38" s="172" t="n"/>
-      <c r="E38" s="172" t="n"/>
-      <c r="F38" s="172" t="n"/>
-      <c r="G38" s="173" t="n"/>
+      <c r="A38" s="125" t="n"/>
+      <c r="B38" s="132" t="n"/>
+      <c r="C38" s="132" t="n"/>
+      <c r="D38" s="132" t="n"/>
+      <c r="E38" s="132" t="n"/>
+      <c r="F38" s="132" t="n"/>
+      <c r="G38" s="155" t="n"/>
+      <c r="H38" s="125" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1" s="101">
-      <c r="B39" s="133" t="n"/>
-      <c r="C39" s="133" t="n"/>
-      <c r="D39" s="133" t="n"/>
-      <c r="E39" s="133" t="n"/>
-      <c r="F39" s="133" t="n"/>
-      <c r="G39" s="221" t="n"/>
+      <c r="A39" s="125" t="n"/>
+      <c r="B39" s="170" t="n"/>
+      <c r="C39" s="170" t="n"/>
+      <c r="D39" s="170" t="n"/>
+      <c r="E39" s="170" t="n"/>
+      <c r="F39" s="170" t="n"/>
+      <c r="G39" s="171" t="n"/>
+      <c r="H39" s="125" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1" s="101">
-      <c r="B40" s="172" t="n"/>
-      <c r="C40" s="172" t="n"/>
-      <c r="D40" s="172" t="n"/>
-      <c r="E40" s="172" t="n"/>
-      <c r="F40" s="172" t="n"/>
-      <c r="G40" s="173" t="n"/>
+      <c r="A40" s="125" t="n"/>
+      <c r="B40" s="132" t="n"/>
+      <c r="C40" s="132" t="n"/>
+      <c r="D40" s="132" t="n"/>
+      <c r="E40" s="132" t="n"/>
+      <c r="F40" s="132" t="n"/>
+      <c r="G40" s="155" t="n"/>
+      <c r="H40" s="125" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1" s="101">
-      <c r="B41" s="133" t="n"/>
-      <c r="C41" s="133" t="n"/>
-      <c r="D41" s="133" t="n"/>
-      <c r="E41" s="133" t="n"/>
-      <c r="F41" s="133" t="n"/>
-      <c r="G41" s="221" t="n"/>
+      <c r="A41" s="125" t="n"/>
+      <c r="B41" s="170" t="n"/>
+      <c r="C41" s="170" t="n"/>
+      <c r="D41" s="170" t="n"/>
+      <c r="E41" s="170" t="n"/>
+      <c r="F41" s="170" t="n"/>
+      <c r="G41" s="171" t="n"/>
+      <c r="H41" s="125" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1" s="101">
-      <c r="B42" s="172" t="n"/>
-      <c r="C42" s="172" t="n"/>
-      <c r="D42" s="172" t="n"/>
-      <c r="E42" s="172" t="n"/>
-      <c r="F42" s="172" t="n"/>
-      <c r="G42" s="173" t="n"/>
+      <c r="A42" s="125" t="n"/>
+      <c r="B42" s="132" t="n"/>
+      <c r="C42" s="132" t="n"/>
+      <c r="D42" s="132" t="n"/>
+      <c r="E42" s="132" t="n"/>
+      <c r="F42" s="132" t="n"/>
+      <c r="G42" s="155" t="n"/>
+      <c r="H42" s="125" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1" s="101">
-      <c r="B43" s="133" t="n"/>
-      <c r="C43" s="133" t="n"/>
-      <c r="D43" s="133" t="n"/>
-      <c r="E43" s="133" t="n"/>
-      <c r="F43" s="133" t="n"/>
-      <c r="G43" s="221" t="n"/>
-    </row>
-    <row r="44" ht="10" customHeight="1" s="101">
-      <c r="B44" s="175" t="inlineStr">
+      <c r="A43" s="125" t="n"/>
+      <c r="B43" s="172" t="inlineStr">
         <is>
           <t>TOTAL OUTROS</t>
         </is>
       </c>
-      <c r="G44" s="176">
+      <c r="G43" s="173">
         <f>SUM(G37:G42)</f>
         <v/>
       </c>
-    </row>
-    <row r="45" ht="26" customHeight="1" s="101"/>
+      <c r="H43" s="125" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="125" t="n"/>
+      <c r="B44" s="125" t="n"/>
+      <c r="C44" s="125" t="n"/>
+      <c r="D44" s="125" t="n"/>
+      <c r="E44" s="125" t="n"/>
+      <c r="F44" s="125" t="n"/>
+      <c r="G44" s="125" t="n"/>
+      <c r="H44" s="125" t="n"/>
+    </row>
+    <row r="45" ht="26" customHeight="1" s="101">
+      <c r="A45" s="125" t="n"/>
+      <c r="B45" s="174" t="inlineStr">
+        <is>
+          <t>RESUMO TOTAL DA VIAGEM</t>
+        </is>
+      </c>
+      <c r="H45" s="125" t="n"/>
+    </row>
     <row r="46" ht="22" customHeight="1" s="101">
-      <c r="B46" s="177" t="inlineStr">
-        <is>
-          <t>💰  RESUMO TOTAL DA VIAGEM</t>
-        </is>
-      </c>
+      <c r="A46" s="125" t="n"/>
+      <c r="B46" s="175" t="inlineStr">
+        <is>
+          <t>Combustivel</t>
+        </is>
+      </c>
+      <c r="G46" s="176">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="H46" s="125" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1" s="101">
-      <c r="B47" s="178" t="inlineStr">
-        <is>
-          <t>⛽ Combustível</t>
-        </is>
-      </c>
-      <c r="G47" s="179">
-        <f>C16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1" s="101">
-      <c r="B48" s="180" t="inlineStr">
-        <is>
-          <t>🏨 Hospedagem</t>
-        </is>
-      </c>
-      <c r="G48" s="181">
+      <c r="A47" s="125" t="n"/>
+      <c r="B47" s="177" t="inlineStr">
+        <is>
+          <t>Hospedagem</t>
+        </is>
+      </c>
+      <c r="G47" s="178">
         <f>G27</f>
         <v/>
       </c>
-    </row>
-    <row r="49" ht="22" customHeight="1" s="101">
-      <c r="B49" s="182" t="inlineStr">
-        <is>
-          <t>🍽️ Alimentação</t>
-        </is>
-      </c>
-      <c r="G49" s="235">
+      <c r="H47" s="125" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1" s="101">
+      <c r="A48" s="125" t="n"/>
+      <c r="B48" s="179" t="inlineStr">
+        <is>
+          <t>Alimentacao</t>
+        </is>
+      </c>
+      <c r="G48" s="180">
         <f>C33</f>
         <v/>
       </c>
-    </row>
-    <row r="50" ht="36" customHeight="1" s="101">
-      <c r="B50" s="184" t="inlineStr">
-        <is>
-          <t>🎡 Outros</t>
-        </is>
-      </c>
-      <c r="G50" s="185">
+      <c r="H48" s="125" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1" s="101">
+      <c r="A49" s="125" t="n"/>
+      <c r="B49" s="181" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="G49" s="182">
         <f>G43</f>
         <v/>
       </c>
-    </row>
-    <row r="51" ht="22" customHeight="1" s="101">
-      <c r="B51" s="186" t="inlineStr">
-        <is>
-          <t>🧳 TOTAL DA VIAGEM</t>
-        </is>
-      </c>
-      <c r="G51" s="187">
+      <c r="H49" s="125" t="n"/>
+    </row>
+    <row r="50" ht="36" customHeight="1" s="101">
+      <c r="A50" s="125" t="n"/>
+      <c r="B50" s="183" t="inlineStr">
+        <is>
+          <t>TOTAL DA VIAGEM</t>
+        </is>
+      </c>
+      <c r="G50" s="184">
         <f>SUM(G46:G49)</f>
         <v/>
       </c>
+      <c r="H50" s="125" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1" s="101">
+      <c r="A51" s="125" t="n"/>
+      <c r="B51" s="185" t="inlineStr">
+        <is>
+          <t>Total por pessoa</t>
+        </is>
+      </c>
+      <c r="G51" s="186">
+        <f>IFERROR(G50/C9,0)</f>
+        <v/>
+      </c>
+      <c r="H51" s="125" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1" s="101">
-      <c r="B52" s="188" t="inlineStr">
-        <is>
-          <t>👤 Total por pessoa</t>
-        </is>
-      </c>
-      <c r="G52" s="189">
-        <f>IFERROR(G50/C7,0)</f>
+      <c r="A52" s="125" t="n"/>
+      <c r="B52" s="187">
+        <f>IF(C10-G50&gt;=0,"Sobra do orcamento","Estouro do orcamento")</f>
         <v/>
       </c>
+      <c r="G52" s="188">
+        <f>C10-G50</f>
+        <v/>
+      </c>
+      <c r="H52" s="125" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="190">
-        <f>IF(C8-G50&gt;=0,"✅ Sobra do orçamento","⚠️ Estouro do orçamento")</f>
-        <v/>
-      </c>
-      <c r="G53" s="191">
-        <f>C8-G50</f>
-        <v/>
-      </c>
+      <c r="A53" s="125" t="n"/>
+      <c r="B53" s="125" t="n"/>
+      <c r="C53" s="125" t="n"/>
+      <c r="D53" s="125" t="n"/>
+      <c r="E53" s="125" t="n"/>
+      <c r="F53" s="125" t="n"/>
+      <c r="G53" s="125" t="n"/>
+      <c r="H53" s="125" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="125" t="n"/>
+      <c r="B54" s="125" t="n"/>
+      <c r="C54" s="125" t="n"/>
+      <c r="D54" s="125" t="n"/>
+      <c r="E54" s="125" t="n"/>
+      <c r="F54" s="125" t="n"/>
+      <c r="G54" s="125" t="n"/>
+      <c r="H54" s="125" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="125" t="n"/>
+      <c r="B55" s="125" t="n"/>
+      <c r="C55" s="125" t="n"/>
+      <c r="D55" s="125" t="n"/>
+      <c r="E55" s="125" t="n"/>
+      <c r="F55" s="125" t="n"/>
+      <c r="G55" s="125" t="n"/>
+      <c r="H55" s="125" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="125" t="n"/>
+      <c r="B56" s="125" t="n"/>
+      <c r="C56" s="125" t="n"/>
+      <c r="D56" s="125" t="n"/>
+      <c r="E56" s="125" t="n"/>
+      <c r="F56" s="125" t="n"/>
+      <c r="G56" s="125" t="n"/>
+      <c r="H56" s="125" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="125" t="n"/>
+      <c r="B57" s="125" t="n"/>
+      <c r="C57" s="125" t="n"/>
+      <c r="D57" s="125" t="n"/>
+      <c r="E57" s="125" t="n"/>
+      <c r="F57" s="125" t="n"/>
+      <c r="G57" s="125" t="n"/>
+      <c r="H57" s="125" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="125" t="n"/>
+      <c r="B58" s="125" t="n"/>
+      <c r="C58" s="125" t="n"/>
+      <c r="D58" s="125" t="n"/>
+      <c r="E58" s="125" t="n"/>
+      <c r="F58" s="125" t="n"/>
+      <c r="G58" s="125" t="n"/>
+      <c r="H58" s="125" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="125" t="n"/>
+      <c r="B59" s="125" t="n"/>
+      <c r="C59" s="125" t="n"/>
+      <c r="D59" s="125" t="n"/>
+      <c r="E59" s="125" t="n"/>
+      <c r="F59" s="125" t="n"/>
+      <c r="G59" s="125" t="n"/>
+      <c r="H59" s="125" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="125" t="n"/>
+      <c r="B60" s="125" t="n"/>
+      <c r="C60" s="125" t="n"/>
+      <c r="D60" s="125" t="n"/>
+      <c r="E60" s="125" t="n"/>
+      <c r="F60" s="125" t="n"/>
+      <c r="G60" s="125" t="n"/>
+      <c r="H60" s="125" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="24">
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="B46:F46"/>
-    <mergeCell ref="D5:G5"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="B29:G29"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B43:F43"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="B20:G20"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="D6:G6"/>
     <mergeCell ref="B45:G45"/>
     <mergeCell ref="B35:G35"/>
-    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E18:G18"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="B3:G3"/>
+    <mergeCell ref="C5:E5"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="C4:E4"/>
     <mergeCell ref="E17:G17"/>
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="D4:G4"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="C37:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Ingresso,Passeio,Transporte,Compras,Emergência,Outro"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C37:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Ingresso,Passeio,Transporte,Compras,Emergência,Outro"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20532,11 +20676,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="101" min="1" max="1"/>
-    <col width="20" customWidth="1" style="101" min="2" max="2"/>
+    <col width="22" customWidth="1" style="101" min="2" max="2"/>
     <col width="8" customWidth="1" style="101" min="3" max="3"/>
     <col width="8" customWidth="1" style="101" min="4" max="4"/>
     <col width="3" customWidth="1" style="101" min="5" max="5"/>
@@ -20546,510 +20690,735 @@
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1" s="101">
-      <c r="A1" s="192" t="inlineStr">
-        <is>
-          <t>🛒  COMPRAS &amp; METAS FINANCEIRAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="10" customHeight="1" s="101"/>
+      <c r="A1" s="189" t="inlineStr">
+        <is>
+          <t>COMPRAS &amp; METAS FINANCEIRAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="125" t="n"/>
+      <c r="B2" s="125" t="n"/>
+      <c r="C2" s="125" t="n"/>
+      <c r="D2" s="125" t="n"/>
+      <c r="E2" s="125" t="n"/>
+      <c r="F2" s="125" t="n"/>
+      <c r="G2" s="125" t="n"/>
+      <c r="H2" s="125" t="n"/>
+    </row>
     <row r="3" ht="28" customHeight="1" s="101">
-      <c r="A3" s="193" t="inlineStr">
-        <is>
-          <t>🎯  CALCULADORA DE META — Quanto guardar por mês</t>
+      <c r="A3" s="190" t="inlineStr">
+        <is>
+          <t>CALCULADORA DE META — Quanto guardar por mes</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" s="101">
-      <c r="A4" s="194" t="inlineStr">
+      <c r="A4" s="160" t="inlineStr">
         <is>
           <t>Produto / Objetivo</t>
         </is>
       </c>
-      <c r="E4" s="195" t="inlineStr"/>
+      <c r="E4" s="191" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1" s="101">
-      <c r="A5" s="194" t="inlineStr">
-        <is>
-          <t>Valor total necessário (R$)</t>
-        </is>
-      </c>
-      <c r="E5" s="196" t="n">
+      <c r="A5" s="137" t="inlineStr">
+        <is>
+          <t>Valor total necessario (R$)</t>
+        </is>
+      </c>
+      <c r="E5" s="156" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" s="101">
-      <c r="A6" s="197" t="inlineStr">
-        <is>
-          <t>Já tenho guardado (R$)</t>
-        </is>
-      </c>
-      <c r="E6" s="196" t="n">
+      <c r="A6" s="160" t="inlineStr">
+        <is>
+          <t>Ja tenho guardado (R$)</t>
+        </is>
+      </c>
+      <c r="E6" s="153" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" s="101">
-      <c r="A7" s="198" t="inlineStr">
-        <is>
-          <t>→ Quanto ainda falta (R$)</t>
-        </is>
-      </c>
-      <c r="E7" s="199">
+      <c r="A7" s="192" t="inlineStr">
+        <is>
+          <t>Quanto falta (R$)</t>
+        </is>
+      </c>
+      <c r="E7" s="193">
         <f>IFERROR(E5-E6,0)</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="10" customHeight="1" s="101">
-      <c r="A8" s="200" t="n"/>
-      <c r="B8" s="200" t="n"/>
-      <c r="C8" s="200" t="n"/>
-      <c r="D8" s="200" t="n"/>
-      <c r="E8" s="200" t="n"/>
-      <c r="F8" s="200" t="n"/>
-      <c r="G8" s="200" t="n"/>
-      <c r="H8" s="200" t="n"/>
+    <row r="8" ht="4" customHeight="1" s="101">
+      <c r="A8" s="194" t="n"/>
+      <c r="B8" s="194" t="n"/>
+      <c r="C8" s="194" t="n"/>
+      <c r="D8" s="194" t="n"/>
+      <c r="E8" s="194" t="n"/>
+      <c r="F8" s="194" t="n"/>
+      <c r="G8" s="194" t="n"/>
+      <c r="H8" s="194" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1" s="101">
-      <c r="A9" s="201" t="inlineStr">
-        <is>
-          <t>📌 OPÇÃO A — Quero comprar em X meses</t>
-        </is>
-      </c>
-      <c r="E9" s="202" t="inlineStr">
-        <is>
-          <t>📌 OPÇÃO B — Consigo guardar X por mês</t>
+      <c r="A9" s="195" t="inlineStr">
+        <is>
+          <t>OPCAO A — Quero comprar em X meses</t>
+        </is>
+      </c>
+      <c r="E9" s="196" t="inlineStr">
+        <is>
+          <t>OPCAO B — Consigo guardar X por mes</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" s="101">
-      <c r="A10" s="203" t="inlineStr">
+      <c r="A10" s="197" t="inlineStr">
         <is>
           <t>Quero comprar em (meses):</t>
         </is>
       </c>
-      <c r="C10" s="204" t="n">
+      <c r="C10" s="198" t="n">
         <v>12</v>
       </c>
-      <c r="E10" s="203" t="inlineStr">
-        <is>
-          <t>Consigo guardar por mês (R$):</t>
-        </is>
-      </c>
-      <c r="G10" s="205" t="n">
+      <c r="E10" s="197" t="inlineStr">
+        <is>
+          <t>Consigo guardar por mes (R$):</t>
+        </is>
+      </c>
+      <c r="G10" s="199" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" s="101">
-      <c r="A11" s="206" t="inlineStr">
-        <is>
-          <t>→ Guardar por mês:</t>
-        </is>
-      </c>
-      <c r="C11" s="207">
+      <c r="A11" s="200" t="inlineStr">
+        <is>
+          <t>Guardar por mes:</t>
+        </is>
+      </c>
+      <c r="C11" s="201">
         <f>IFERROR(E7/C10,0)</f>
         <v/>
       </c>
-      <c r="E11" s="206" t="inlineStr">
-        <is>
-          <t>→ Meses até a compra:</t>
-        </is>
-      </c>
-      <c r="G11" s="208">
+      <c r="E11" s="200" t="inlineStr">
+        <is>
+          <t>Meses ate a compra:</t>
+        </is>
+      </c>
+      <c r="G11" s="202">
         <f>IFERROR(CEILING(E7/G10,1),0)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" s="101">
-      <c r="A12" s="209" t="inlineStr">
-        <is>
-          <t>→ Data estimada (Opção A):</t>
-        </is>
-      </c>
-      <c r="C12" s="210">
+      <c r="A12" s="203" t="inlineStr">
+        <is>
+          <t>Data estimada (Opcao A):</t>
+        </is>
+      </c>
+      <c r="C12" s="204">
         <f>IFERROR(EDATE(TODAY(),C10),"")</f>
         <v/>
       </c>
-      <c r="E12" s="209" t="inlineStr">
-        <is>
-          <t>→ Data estimada (Opção B):</t>
-        </is>
-      </c>
-      <c r="G12" s="211">
+      <c r="E12" s="203" t="inlineStr">
+        <is>
+          <t>Data estimada (Opcao B):</t>
+        </is>
+      </c>
+      <c r="G12" s="205">
         <f>IFERROR(EDATE(TODAY(),G11),"")</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="10" customHeight="1" s="101"/>
+    <row r="13">
+      <c r="A13" s="125" t="n"/>
+      <c r="B13" s="125" t="n"/>
+      <c r="C13" s="125" t="n"/>
+      <c r="D13" s="125" t="n"/>
+      <c r="E13" s="125" t="n"/>
+      <c r="F13" s="125" t="n"/>
+      <c r="G13" s="125" t="n"/>
+      <c r="H13" s="125" t="n"/>
+    </row>
     <row r="14" ht="26" customHeight="1" s="101">
-      <c r="A14" s="212" t="inlineStr">
-        <is>
-          <t>📋  LISTA DE METAS DE COMPRA</t>
+      <c r="A14" s="206" t="inlineStr">
+        <is>
+          <t>LISTA DE METAS DE COMPRA</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" s="101">
-      <c r="A15" s="213" t="inlineStr">
+      <c r="A15" s="150" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B15" s="213" t="inlineStr">
+      <c r="B15" s="150" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="C15" s="213" t="inlineStr">
-        <is>
-          <t>Valor (R$)</t>
-        </is>
-      </c>
-      <c r="D15" s="213" t="inlineStr">
-        <is>
-          <t>Guardado (R$)</t>
-        </is>
-      </c>
-      <c r="E15" s="213" t="inlineStr">
-        <is>
-          <t>Falta (R$)</t>
-        </is>
-      </c>
-      <c r="F15" s="213" t="inlineStr">
-        <is>
-          <t>Poupar/mês</t>
-        </is>
-      </c>
-      <c r="G15" s="213" t="inlineStr">
+      <c r="C15" s="150" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="D15" s="150" t="inlineStr">
+        <is>
+          <t>Guardado</t>
+        </is>
+      </c>
+      <c r="E15" s="150" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F15" s="150" t="inlineStr">
+        <is>
+          <t>Poupar/mes</t>
+        </is>
+      </c>
+      <c r="G15" s="150" t="inlineStr">
         <is>
           <t>Meses</t>
         </is>
       </c>
-      <c r="H15" s="213" t="inlineStr">
-        <is>
-          <t>Previsão</t>
+      <c r="H15" s="150" t="inlineStr">
+        <is>
+          <t>Previsao</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" s="101">
-      <c r="A16" s="214" t="n">
+      <c r="A16" s="207" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="135" t="n"/>
-      <c r="C16" s="215" t="n"/>
-      <c r="D16" s="215" t="n"/>
-      <c r="E16" s="216">
+      <c r="B16" s="130" t="n"/>
+      <c r="C16" s="208" t="n"/>
+      <c r="D16" s="208" t="n"/>
+      <c r="E16" s="209">
         <f>IFERROR(C16-D16,0)</f>
         <v/>
       </c>
-      <c r="F16" s="217">
+      <c r="F16" s="210">
         <f>IFERROR(E16/C10,0)</f>
         <v/>
       </c>
-      <c r="G16" s="218">
+      <c r="G16" s="211">
         <f>IFERROR(CEILING(E16/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H16" s="219">
+      <c r="H16" s="212">
         <f>IFERROR(EDATE(TODAY(),G16),"")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" s="101">
-      <c r="A17" s="220" t="n">
+      <c r="A17" s="213" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="133" t="n"/>
-      <c r="C17" s="221" t="n"/>
-      <c r="D17" s="221" t="n"/>
-      <c r="E17" s="222">
+      <c r="B17" s="132" t="n"/>
+      <c r="C17" s="214" t="n"/>
+      <c r="D17" s="214" t="n"/>
+      <c r="E17" s="215">
         <f>IFERROR(C17-D17,0)</f>
         <v/>
       </c>
-      <c r="F17" s="223">
+      <c r="F17" s="216">
         <f>IFERROR(E17/C10,0)</f>
         <v/>
       </c>
-      <c r="G17" s="224">
+      <c r="G17" s="217">
         <f>IFERROR(CEILING(E17/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H17" s="225">
+      <c r="H17" s="218">
         <f>IFERROR(EDATE(TODAY(),G17),"")</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" s="101">
-      <c r="A18" s="214" t="n">
+      <c r="A18" s="207" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="135" t="n"/>
-      <c r="C18" s="215" t="n"/>
-      <c r="D18" s="215" t="n"/>
-      <c r="E18" s="216">
+      <c r="B18" s="130" t="n"/>
+      <c r="C18" s="208" t="n"/>
+      <c r="D18" s="208" t="n"/>
+      <c r="E18" s="209">
         <f>IFERROR(C18-D18,0)</f>
         <v/>
       </c>
-      <c r="F18" s="217">
+      <c r="F18" s="210">
         <f>IFERROR(E18/C10,0)</f>
         <v/>
       </c>
-      <c r="G18" s="218">
+      <c r="G18" s="211">
         <f>IFERROR(CEILING(E18/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H18" s="219">
+      <c r="H18" s="212">
         <f>IFERROR(EDATE(TODAY(),G18),"")</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" s="101">
-      <c r="A19" s="220" t="n">
+      <c r="A19" s="213" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="133" t="n"/>
-      <c r="C19" s="221" t="n"/>
-      <c r="D19" s="221" t="n"/>
-      <c r="E19" s="222">
+      <c r="B19" s="132" t="n"/>
+      <c r="C19" s="214" t="n"/>
+      <c r="D19" s="214" t="n"/>
+      <c r="E19" s="215">
         <f>IFERROR(C19-D19,0)</f>
         <v/>
       </c>
-      <c r="F19" s="223">
+      <c r="F19" s="216">
         <f>IFERROR(E19/C10,0)</f>
         <v/>
       </c>
-      <c r="G19" s="224">
+      <c r="G19" s="217">
         <f>IFERROR(CEILING(E19/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H19" s="225">
+      <c r="H19" s="218">
         <f>IFERROR(EDATE(TODAY(),G19),"")</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" s="101">
-      <c r="A20" s="214" t="n">
+      <c r="A20" s="207" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="135" t="n"/>
-      <c r="C20" s="215" t="n"/>
-      <c r="D20" s="215" t="n"/>
-      <c r="E20" s="216">
+      <c r="B20" s="130" t="n"/>
+      <c r="C20" s="208" t="n"/>
+      <c r="D20" s="208" t="n"/>
+      <c r="E20" s="209">
         <f>IFERROR(C20-D20,0)</f>
         <v/>
       </c>
-      <c r="F20" s="217">
+      <c r="F20" s="210">
         <f>IFERROR(E20/C10,0)</f>
         <v/>
       </c>
-      <c r="G20" s="218">
+      <c r="G20" s="211">
         <f>IFERROR(CEILING(E20/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H20" s="219">
+      <c r="H20" s="212">
         <f>IFERROR(EDATE(TODAY(),G20),"")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" s="101">
-      <c r="A21" s="220" t="n">
+      <c r="A21" s="213" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="133" t="n"/>
-      <c r="C21" s="221" t="n"/>
-      <c r="D21" s="221" t="n"/>
-      <c r="E21" s="222">
+      <c r="B21" s="132" t="n"/>
+      <c r="C21" s="214" t="n"/>
+      <c r="D21" s="214" t="n"/>
+      <c r="E21" s="215">
         <f>IFERROR(C21-D21,0)</f>
         <v/>
       </c>
-      <c r="F21" s="223">
+      <c r="F21" s="216">
         <f>IFERROR(E21/C10,0)</f>
         <v/>
       </c>
-      <c r="G21" s="224">
+      <c r="G21" s="217">
         <f>IFERROR(CEILING(E21/G10,1),0)</f>
         <v/>
       </c>
-      <c r="H21" s="225">
+      <c r="H21" s="218">
         <f>IFERROR(EDATE(TODAY(),G21),"")</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="14" customHeight="1" s="101"/>
+    <row r="22">
+      <c r="A22" s="125" t="n"/>
+      <c r="B22" s="125" t="n"/>
+      <c r="C22" s="125" t="n"/>
+      <c r="D22" s="125" t="n"/>
+      <c r="E22" s="125" t="n"/>
+      <c r="F22" s="125" t="n"/>
+      <c r="G22" s="125" t="n"/>
+      <c r="H22" s="125" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="125" t="n"/>
+      <c r="B23" s="125" t="n"/>
+      <c r="C23" s="125" t="n"/>
+      <c r="D23" s="125" t="n"/>
+      <c r="E23" s="125" t="n"/>
+      <c r="F23" s="125" t="n"/>
+      <c r="G23" s="125" t="n"/>
+      <c r="H23" s="125" t="n"/>
+    </row>
     <row r="24" ht="28" customHeight="1" s="101">
-      <c r="A24" s="226" t="inlineStr">
-        <is>
-          <t>💳  CALCULADORA: À VISTA vs PARCELADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="14" customHeight="1" s="101">
-      <c r="A25" s="227" t="inlineStr">
-        <is>
-          <t>Preencha os campos em AZUL — o restante é calculado automaticamente</t>
-        </is>
-      </c>
+      <c r="A24" s="219" t="inlineStr">
+        <is>
+          <t>CALCULADORA: A VISTA vs PARCELADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="101">
+      <c r="A25" s="137" t="inlineStr">
+        <is>
+          <t>Produto / Descricao</t>
+        </is>
+      </c>
+      <c r="E25" s="220" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1" s="101">
-      <c r="A26" s="197" t="inlineStr">
-        <is>
-          <t>Produto / Descrição</t>
-        </is>
-      </c>
-      <c r="E26" s="228" t="inlineStr"/>
+      <c r="A26" s="160" t="inlineStr">
+        <is>
+          <t>Preco a VISTA (R$)</t>
+        </is>
+      </c>
+      <c r="E26" s="221" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="22" customHeight="1" s="101">
-      <c r="A27" s="229" t="inlineStr">
-        <is>
-          <t>Preço à VISTA (R$)</t>
-        </is>
-      </c>
-      <c r="E27" s="230" t="n">
+      <c r="A27" s="137" t="inlineStr">
+        <is>
+          <t>Desconto a vista (%)</t>
+        </is>
+      </c>
+      <c r="E27" s="220" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" s="101">
-      <c r="A28" s="197" t="inlineStr">
-        <is>
-          <t>Desconto à vista (%)</t>
-        </is>
-      </c>
-      <c r="E28" s="231" t="n">
+      <c r="A28" s="222" t="inlineStr">
+        <is>
+          <t>Preco a vista c/ desconto</t>
+        </is>
+      </c>
+      <c r="E28" s="223">
+        <f>IFERROR(E26*(1-E27/100),E26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="101">
+      <c r="A29" s="137" t="inlineStr">
+        <is>
+          <t>Numero de parcelas</t>
+        </is>
+      </c>
+      <c r="E29" s="220" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" s="101">
+      <c r="A30" s="160" t="inlineStr">
+        <is>
+          <t>Valor de cada parcela (R$)</t>
+        </is>
+      </c>
+      <c r="E30" s="221" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1" s="101">
-      <c r="A29" s="232" t="inlineStr">
-        <is>
-          <t>→ Preço à vista c/ desconto</t>
-        </is>
-      </c>
-      <c r="E29" s="233">
-        <f>IFERROR(E27*(1-E28/100),E27)</f>
+    <row r="31" ht="6" customHeight="1" s="101">
+      <c r="A31" s="194" t="n"/>
+      <c r="B31" s="194" t="n"/>
+      <c r="C31" s="194" t="n"/>
+      <c r="D31" s="194" t="n"/>
+      <c r="E31" s="194" t="n"/>
+      <c r="F31" s="194" t="n"/>
+      <c r="G31" s="194" t="n"/>
+      <c r="H31" s="194" t="n"/>
+    </row>
+    <row r="32" ht="24" customHeight="1" s="101">
+      <c r="A32" s="206" t="inlineStr">
+        <is>
+          <t>ANALISE COMPARATIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="101">
+      <c r="A33" s="137" t="inlineStr">
+        <is>
+          <t>Total pago a vista</t>
+        </is>
+      </c>
+      <c r="E33" s="224">
+        <f>IFERROR(E28,E26)</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1" s="101">
-      <c r="A30" s="197" t="inlineStr">
-        <is>
-          <t>Número de parcelas</t>
-        </is>
-      </c>
-      <c r="E30" s="234" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" s="101">
-      <c r="A31" s="229" t="inlineStr">
-        <is>
-          <t>Valor de cada parcela (R$)</t>
-        </is>
-      </c>
-      <c r="E31" s="230" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="8" customHeight="1" s="101">
-      <c r="A32" s="200" t="n"/>
-      <c r="B32" s="200" t="n"/>
-      <c r="C32" s="200" t="n"/>
-      <c r="D32" s="200" t="n"/>
-      <c r="E32" s="200" t="n"/>
-      <c r="F32" s="200" t="n"/>
-      <c r="G32" s="200" t="n"/>
-      <c r="H32" s="200" t="n"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" s="101">
-      <c r="A33" s="212" t="inlineStr">
-        <is>
-          <t>📊  ANÁLISE COMPARATIVA</t>
-        </is>
-      </c>
-    </row>
     <row r="34" ht="22" customHeight="1" s="101">
-      <c r="A34" s="197" t="inlineStr">
-        <is>
-          <t>💵 Total pago à vista</t>
-        </is>
-      </c>
-      <c r="E34" s="235">
-        <f>IFERROR(E29,E27)</f>
+      <c r="A34" s="160" t="inlineStr">
+        <is>
+          <t>Total pago parcelado</t>
+        </is>
+      </c>
+      <c r="E34" s="225">
+        <f>IFERROR(E29*E30,0)</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1" s="101">
-      <c r="A35" s="229" t="inlineStr">
-        <is>
-          <t>💳 Total pago parcelado</t>
-        </is>
-      </c>
-      <c r="E35" s="236">
-        <f>IFERROR(E30*E31,0)</f>
+    <row r="35" ht="24" customHeight="1" s="101">
+      <c r="A35" s="226" t="inlineStr">
+        <is>
+          <t>Quanto a mais no parcelado (R$)</t>
+        </is>
+      </c>
+      <c r="E35" s="227">
+        <f>IFERROR(E34-E33,0)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="101">
-      <c r="A36" s="237" t="inlineStr">
-        <is>
-          <t>📈 Quanto a mais no parcelado (R$)</t>
-        </is>
-      </c>
-      <c r="E36" s="238">
-        <f>IFERROR(E35-E34,0)</f>
+      <c r="A36" s="226" t="inlineStr">
+        <is>
+          <t>Quanto a mais no parcelado (%)</t>
+        </is>
+      </c>
+      <c r="E36" s="228">
+        <f>IFERROR((E34/E33-1)*100,0)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1" s="101">
-      <c r="A37" s="237" t="inlineStr">
-        <is>
-          <t>📈 Quanto a mais no parcelado (%)</t>
-        </is>
-      </c>
-      <c r="E37" s="239">
-        <f>IFERROR((E35/E34-1)*100,0)</f>
+      <c r="A37" s="226" t="inlineStr">
+        <is>
+          <t>Taxa de juros mensal (RATE)</t>
+        </is>
+      </c>
+      <c r="E37" s="229">
+        <f>IFERROR(RATE(E29,-E30,E28)*100,0)</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" s="101">
-      <c r="A38" s="237" t="inlineStr">
-        <is>
-          <t>🔢 Taxa de juros mensal (RATE)</t>
-        </is>
-      </c>
-      <c r="E38" s="240">
-        <f>IFERROR(RATE(E30,-E31,E29)*100,0)</f>
+      <c r="A38" s="226" t="inlineStr">
+        <is>
+          <t>Taxa de juros anual equivalente</t>
+        </is>
+      </c>
+      <c r="E38" s="229">
+        <f>IFERROR(((1+E37/100)^12-1)*100,0)</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1" s="101">
-      <c r="A39" s="237" t="inlineStr">
-        <is>
-          <t>🔢 Taxa de juros anual equivalente</t>
-        </is>
-      </c>
-      <c r="E39" s="240">
-        <f>IFERROR(((1+E38/100)^12-1)*100,0)</f>
+    <row r="39">
+      <c r="A39" s="125" t="n"/>
+      <c r="B39" s="125" t="n"/>
+      <c r="C39" s="125" t="n"/>
+      <c r="D39" s="125" t="n"/>
+      <c r="E39" s="125" t="n"/>
+      <c r="F39" s="125" t="n"/>
+      <c r="G39" s="125" t="n"/>
+      <c r="H39" s="125" t="n"/>
+    </row>
+    <row r="40" ht="48" customHeight="1" s="101">
+      <c r="A40" s="230">
+        <f>IFERROR(IF(E37&lt;=0,"Preencha preco a vista e valor da parcela",IF(E37&lt;0.8,"JUROS BAIXOS ("&amp;TEXT(E37,"0.00")&amp;"% a.m.) — Parcelar pode valer se voce investir a diferenca",IF(E37&lt;1.5,"JUROS MODERADOS ("&amp;TEXT(E37,"0.00")&amp;"% a.m.) — Prefira a vista se possivel",IF(E37&lt;3,"JUROS ALTOS ("&amp;TEXT(E37,"0.00")&amp;"% a.m.) — Compre A VISTA. Parcelado custa "&amp;TEXT(E35,"R$ #,##0.00")&amp;" a mais","JUROS ABUSIVOS ("&amp;TEXT(E37,"0.00")&amp;"% a.m.) — NUNCA parcele nessas condicoes!")))),"")</f>
         <v/>
       </c>
     </row>
-    <row r="40" ht="10" customHeight="1" s="101"/>
-    <row r="41" ht="40" customHeight="1" s="101">
-      <c r="A41" s="241">
-        <f>IFERROR(IF(E38&lt;=0,"⚠️ Preencha preço à vista e valor da parcela",
-IF(E38&lt;0.8,"✅ JUROS BAIXOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Parcelar pode valer se você investir a diferença",
-IF(E38&lt;1.5,"⚡ JUROS MODERADOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Prefira à vista se possível",
-IF(E38&lt;3,"🔴 JUROS ALTOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — Compre À VISTA. Parcelado custa "&amp;TEXT(E36,"R$ #,##0.00")&amp;" a mais",
-"🚨 JUROS ABUSIVOS ("&amp;TEXT(E38,"0.00")&amp;"% a.m.) — NUNCA parcele nessas condições!")))),"Preencha os dados")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1" s="101">
-      <c r="A42" s="242" t="inlineStr">
-        <is>
-          <t>💡 Dica: Se os juros forem menores que o rendimento da sua reserva (ex: CDB/Tesouro ~0,8%/mês), pode valer guardar o dinheiro e parcelar. Mas se não tiver disciplina, pague à vista.</t>
-        </is>
-      </c>
+    <row r="41" ht="28" customHeight="1" s="101">
+      <c r="A41" s="231" t="inlineStr">
+        <is>
+          <t>Dica: Se os juros forem menores que o rendimento da sua reserva (ex: CDB/Tesouro ~0,8%/mes), pode valer guardar o dinheiro e parcelar. Se nao tiver disciplina, pague a vista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="125" t="n"/>
+      <c r="B42" s="125" t="n"/>
+      <c r="C42" s="125" t="n"/>
+      <c r="D42" s="125" t="n"/>
+      <c r="E42" s="125" t="n"/>
+      <c r="F42" s="125" t="n"/>
+      <c r="G42" s="125" t="n"/>
+      <c r="H42" s="125" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="125" t="n"/>
+      <c r="B43" s="125" t="n"/>
+      <c r="C43" s="125" t="n"/>
+      <c r="D43" s="125" t="n"/>
+      <c r="E43" s="125" t="n"/>
+      <c r="F43" s="125" t="n"/>
+      <c r="G43" s="125" t="n"/>
+      <c r="H43" s="125" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="125" t="n"/>
+      <c r="B44" s="125" t="n"/>
+      <c r="C44" s="125" t="n"/>
+      <c r="D44" s="125" t="n"/>
+      <c r="E44" s="125" t="n"/>
+      <c r="F44" s="125" t="n"/>
+      <c r="G44" s="125" t="n"/>
+      <c r="H44" s="125" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="125" t="n"/>
+      <c r="B45" s="125" t="n"/>
+      <c r="C45" s="125" t="n"/>
+      <c r="D45" s="125" t="n"/>
+      <c r="E45" s="125" t="n"/>
+      <c r="F45" s="125" t="n"/>
+      <c r="G45" s="125" t="n"/>
+      <c r="H45" s="125" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="125" t="n"/>
+      <c r="B46" s="125" t="n"/>
+      <c r="C46" s="125" t="n"/>
+      <c r="D46" s="125" t="n"/>
+      <c r="E46" s="125" t="n"/>
+      <c r="F46" s="125" t="n"/>
+      <c r="G46" s="125" t="n"/>
+      <c r="H46" s="125" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="125" t="n"/>
+      <c r="B47" s="125" t="n"/>
+      <c r="C47" s="125" t="n"/>
+      <c r="D47" s="125" t="n"/>
+      <c r="E47" s="125" t="n"/>
+      <c r="F47" s="125" t="n"/>
+      <c r="G47" s="125" t="n"/>
+      <c r="H47" s="125" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="125" t="n"/>
+      <c r="B48" s="125" t="n"/>
+      <c r="C48" s="125" t="n"/>
+      <c r="D48" s="125" t="n"/>
+      <c r="E48" s="125" t="n"/>
+      <c r="F48" s="125" t="n"/>
+      <c r="G48" s="125" t="n"/>
+      <c r="H48" s="125" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="125" t="n"/>
+      <c r="B49" s="125" t="n"/>
+      <c r="C49" s="125" t="n"/>
+      <c r="D49" s="125" t="n"/>
+      <c r="E49" s="125" t="n"/>
+      <c r="F49" s="125" t="n"/>
+      <c r="G49" s="125" t="n"/>
+      <c r="H49" s="125" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="125" t="n"/>
+      <c r="B50" s="125" t="n"/>
+      <c r="C50" s="125" t="n"/>
+      <c r="D50" s="125" t="n"/>
+      <c r="E50" s="125" t="n"/>
+      <c r="F50" s="125" t="n"/>
+      <c r="G50" s="125" t="n"/>
+      <c r="H50" s="125" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="125" t="n"/>
+      <c r="B51" s="125" t="n"/>
+      <c r="C51" s="125" t="n"/>
+      <c r="D51" s="125" t="n"/>
+      <c r="E51" s="125" t="n"/>
+      <c r="F51" s="125" t="n"/>
+      <c r="G51" s="125" t="n"/>
+      <c r="H51" s="125" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="125" t="n"/>
+      <c r="B52" s="125" t="n"/>
+      <c r="C52" s="125" t="n"/>
+      <c r="D52" s="125" t="n"/>
+      <c r="E52" s="125" t="n"/>
+      <c r="F52" s="125" t="n"/>
+      <c r="G52" s="125" t="n"/>
+      <c r="H52" s="125" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="125" t="n"/>
+      <c r="B53" s="125" t="n"/>
+      <c r="C53" s="125" t="n"/>
+      <c r="D53" s="125" t="n"/>
+      <c r="E53" s="125" t="n"/>
+      <c r="F53" s="125" t="n"/>
+      <c r="G53" s="125" t="n"/>
+      <c r="H53" s="125" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="125" t="n"/>
+      <c r="B54" s="125" t="n"/>
+      <c r="C54" s="125" t="n"/>
+      <c r="D54" s="125" t="n"/>
+      <c r="E54" s="125" t="n"/>
+      <c r="F54" s="125" t="n"/>
+      <c r="G54" s="125" t="n"/>
+      <c r="H54" s="125" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="125" t="n"/>
+      <c r="B55" s="125" t="n"/>
+      <c r="C55" s="125" t="n"/>
+      <c r="D55" s="125" t="n"/>
+      <c r="E55" s="125" t="n"/>
+      <c r="F55" s="125" t="n"/>
+      <c r="G55" s="125" t="n"/>
+      <c r="H55" s="125" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="125" t="n"/>
+      <c r="B56" s="125" t="n"/>
+      <c r="C56" s="125" t="n"/>
+      <c r="D56" s="125" t="n"/>
+      <c r="E56" s="125" t="n"/>
+      <c r="F56" s="125" t="n"/>
+      <c r="G56" s="125" t="n"/>
+      <c r="H56" s="125" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="125" t="n"/>
+      <c r="B57" s="125" t="n"/>
+      <c r="C57" s="125" t="n"/>
+      <c r="D57" s="125" t="n"/>
+      <c r="E57" s="125" t="n"/>
+      <c r="F57" s="125" t="n"/>
+      <c r="G57" s="125" t="n"/>
+      <c r="H57" s="125" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="125" t="n"/>
+      <c r="B58" s="125" t="n"/>
+      <c r="C58" s="125" t="n"/>
+      <c r="D58" s="125" t="n"/>
+      <c r="E58" s="125" t="n"/>
+      <c r="F58" s="125" t="n"/>
+      <c r="G58" s="125" t="n"/>
+      <c r="H58" s="125" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="125" t="n"/>
+      <c r="B59" s="125" t="n"/>
+      <c r="C59" s="125" t="n"/>
+      <c r="D59" s="125" t="n"/>
+      <c r="E59" s="125" t="n"/>
+      <c r="F59" s="125" t="n"/>
+      <c r="G59" s="125" t="n"/>
+      <c r="H59" s="125" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="125" t="n"/>
+      <c r="B60" s="125" t="n"/>
+      <c r="C60" s="125" t="n"/>
+      <c r="D60" s="125" t="n"/>
+      <c r="E60" s="125" t="n"/>
+      <c r="F60" s="125" t="n"/>
+      <c r="G60" s="125" t="n"/>
+      <c r="H60" s="125" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="54">
+  <mergeCells count="53">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="G12:H12"/>
@@ -21062,46 +21431,45 @@
     <mergeCell ref="A38:D38"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E25:H25"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="E37:H37"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A31:D31"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A39:D39"/>
     <mergeCell ref="A41:H41"/>
+    <mergeCell ref="E33:H33"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="A36:D36"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="E39:H39"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="E38:H38"/>
-    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="E29:H29"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="E28:H28"/>
+    <mergeCell ref="A40:H40"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="E9:H9"/>
-    <mergeCell ref="E31:H31"/>
     <mergeCell ref="E34:H34"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="E6:H6"/>
     <mergeCell ref="E30:H30"/>
+    <mergeCell ref="A33:D33"/>
     <mergeCell ref="E27:H27"/>
     <mergeCell ref="E36:H36"/>
   </mergeCells>

</xml_diff>